<commit_message>
update report guidelines, add icons
</commit_message>
<xml_diff>
--- a/analytics/CapstoneDatabase.xlsx
+++ b/analytics/CapstoneDatabase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ernesto/github/MHACapstone/analytics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD0ED93-C8D0-7A4A-800F-BA71E0AFA46F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE5D31D-ABA5-9B43-9697-76AE4D6F65C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="25620" windowHeight="28180" xr2:uid="{DF6E0216-7FF7-48A9-8432-AB69252F5C13}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28180" xr2:uid="{DF6E0216-7FF7-48A9-8432-AB69252F5C13}"/>
   </bookViews>
   <sheets>
     <sheet name="AssetDatabase" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="1001">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="1002">
   <si>
     <t>year</t>
   </si>
@@ -3049,6 +3049,9 @@
   </si>
   <si>
     <t>Lucas</t>
+  </si>
+  <si>
+    <t>Cory Christiansen</t>
   </si>
 </sst>
 </file>
@@ -3593,6 +3596,24 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -3656,24 +3677,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5827,15 +5830,15 @@
       <c r="C28" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="D28" s="56" t="s">
+      <c r="D28" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="58"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="62"/>
+      <c r="G28" s="62"/>
+      <c r="H28" s="62"/>
+      <c r="I28" s="62"/>
+      <c r="J28" s="63"/>
     </row>
     <row r="29" spans="1:117" s="5" customFormat="1" ht="40" x14ac:dyDescent="0.2">
       <c r="A29" s="16">
@@ -6951,7 +6954,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:117" ht="40" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:117" ht="20" x14ac:dyDescent="0.2">
       <c r="A45" s="5">
         <v>2017</v>
       </c>
@@ -7281,15 +7284,15 @@
       <c r="C55" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="D55" s="53" t="s">
+      <c r="D55" s="58" t="s">
         <v>237</v>
       </c>
-      <c r="E55" s="54"/>
-      <c r="F55" s="54"/>
-      <c r="G55" s="54"/>
-      <c r="H55" s="54"/>
-      <c r="I55" s="54"/>
-      <c r="J55" s="55"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="60"/>
     </row>
     <row r="56" spans="1:117" s="5" customFormat="1" ht="20" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
@@ -12342,7 +12345,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="40" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" ht="20" x14ac:dyDescent="0.2">
       <c r="A165" s="16">
         <v>2022</v>
       </c>
@@ -12487,7 +12490,7 @@
         <v>84</v>
       </c>
       <c r="F169" s="5" t="s">
-        <v>39</v>
+        <v>1001</v>
       </c>
       <c r="G169" s="5" t="s">
         <v>674</v>
@@ -13378,22 +13381,22 @@
       <c r="A198" s="2">
         <v>2025</v>
       </c>
-      <c r="B198" s="71" t="s">
+      <c r="B198" s="53" t="s">
         <v>922</v>
       </c>
-      <c r="C198" s="71" t="s">
+      <c r="C198" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="D198" s="71" t="s">
+      <c r="D198" s="53" t="s">
         <v>940</v>
       </c>
-      <c r="E198" s="71" t="s">
+      <c r="E198" s="53" t="s">
         <v>182</v>
       </c>
-      <c r="F198" s="71" t="s">
+      <c r="F198" s="53" t="s">
         <v>941</v>
       </c>
-      <c r="G198" s="71" t="s">
+      <c r="G198" s="53" t="s">
         <v>960</v>
       </c>
       <c r="H198" s="2" t="s">
@@ -13404,22 +13407,22 @@
       <c r="A199" s="2">
         <v>2025</v>
       </c>
-      <c r="B199" s="72" t="s">
+      <c r="B199" s="54" t="s">
         <v>923</v>
       </c>
-      <c r="C199" s="72" t="s">
+      <c r="C199" s="54" t="s">
         <v>924</v>
       </c>
-      <c r="D199" s="72" t="s">
+      <c r="D199" s="54" t="s">
         <v>942</v>
       </c>
-      <c r="E199" s="72" t="s">
+      <c r="E199" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F199" s="72" t="s">
+      <c r="F199" s="54" t="s">
         <v>943</v>
       </c>
-      <c r="G199" s="72" t="s">
+      <c r="G199" s="54" t="s">
         <v>84</v>
       </c>
       <c r="H199" s="2" t="s">
@@ -13430,22 +13433,22 @@
       <c r="A200" s="2">
         <v>2025</v>
       </c>
-      <c r="B200" s="71" t="s">
+      <c r="B200" s="53" t="s">
         <v>925</v>
       </c>
-      <c r="C200" s="71" t="s">
+      <c r="C200" s="53" t="s">
         <v>967</v>
       </c>
-      <c r="D200" s="71" t="s">
+      <c r="D200" s="53" t="s">
         <v>944</v>
       </c>
-      <c r="E200" s="71" t="s">
+      <c r="E200" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="F200" s="71" t="s">
+      <c r="F200" s="53" t="s">
         <v>453</v>
       </c>
-      <c r="G200" s="71" t="s">
+      <c r="G200" s="53" t="s">
         <v>961</v>
       </c>
       <c r="H200" s="2" t="s">
@@ -13456,22 +13459,22 @@
       <c r="A201" s="2">
         <v>2025</v>
       </c>
-      <c r="B201" s="72" t="s">
+      <c r="B201" s="54" t="s">
         <v>926</v>
       </c>
-      <c r="C201" s="72" t="s">
+      <c r="C201" s="54" t="s">
         <v>927</v>
       </c>
-      <c r="D201" s="72" t="s">
+      <c r="D201" s="54" t="s">
         <v>945</v>
       </c>
-      <c r="E201" s="72" t="s">
+      <c r="E201" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F201" s="72" t="s">
+      <c r="F201" s="54" t="s">
         <v>631</v>
       </c>
-      <c r="G201" s="72" t="s">
+      <c r="G201" s="54" t="s">
         <v>962</v>
       </c>
       <c r="H201" s="2" t="s">
@@ -13482,22 +13485,22 @@
       <c r="A202" s="2">
         <v>2025</v>
       </c>
-      <c r="B202" s="71" t="s">
+      <c r="B202" s="53" t="s">
         <v>367</v>
       </c>
-      <c r="C202" s="71" t="s">
+      <c r="C202" s="53" t="s">
         <v>928</v>
       </c>
-      <c r="D202" s="71" t="s">
+      <c r="D202" s="53" t="s">
         <v>946</v>
       </c>
-      <c r="E202" s="71" t="s">
+      <c r="E202" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F202" s="71" t="s">
+      <c r="F202" s="53" t="s">
         <v>302</v>
       </c>
-      <c r="G202" s="71" t="s">
+      <c r="G202" s="53" t="s">
         <v>963</v>
       </c>
       <c r="H202" s="2" t="s">
@@ -13508,22 +13511,22 @@
       <c r="A203" s="2">
         <v>2025</v>
       </c>
-      <c r="B203" s="72" t="s">
+      <c r="B203" s="54" t="s">
         <v>968</v>
       </c>
-      <c r="C203" s="72" t="s">
+      <c r="C203" s="54" t="s">
         <v>596</v>
       </c>
-      <c r="D203" s="72" t="s">
+      <c r="D203" s="54" t="s">
         <v>947</v>
       </c>
-      <c r="E203" s="72" t="s">
+      <c r="E203" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F203" s="72" t="s">
+      <c r="F203" s="54" t="s">
         <v>583</v>
       </c>
-      <c r="G203" s="72" t="s">
+      <c r="G203" s="54" t="s">
         <v>727</v>
       </c>
       <c r="H203" s="2" t="s">
@@ -13534,22 +13537,22 @@
       <c r="A204" s="2">
         <v>2025</v>
       </c>
-      <c r="B204" s="71" t="s">
+      <c r="B204" s="53" t="s">
         <v>929</v>
       </c>
-      <c r="C204" s="71" t="s">
+      <c r="C204" s="53" t="s">
         <v>969</v>
       </c>
-      <c r="D204" s="71" t="s">
+      <c r="D204" s="53" t="s">
         <v>948</v>
       </c>
-      <c r="E204" s="71" t="s">
+      <c r="E204" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="F204" s="71" t="s">
+      <c r="F204" s="53" t="s">
         <v>468</v>
       </c>
-      <c r="G204" s="71" t="s">
+      <c r="G204" s="53" t="s">
         <v>84</v>
       </c>
       <c r="H204" s="2" t="s">
@@ -13560,22 +13563,22 @@
       <c r="A205" s="2">
         <v>2025</v>
       </c>
-      <c r="B205" s="72" t="s">
+      <c r="B205" s="54" t="s">
         <v>930</v>
       </c>
-      <c r="C205" s="72" t="s">
+      <c r="C205" s="54" t="s">
         <v>931</v>
       </c>
-      <c r="D205" s="72" t="s">
+      <c r="D205" s="54" t="s">
         <v>949</v>
       </c>
-      <c r="E205" s="72" t="s">
+      <c r="E205" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F205" s="72" t="s">
+      <c r="F205" s="54" t="s">
         <v>704</v>
       </c>
-      <c r="G205" s="72" t="s">
+      <c r="G205" s="54" t="s">
         <v>964</v>
       </c>
       <c r="H205" s="2" t="s">
@@ -13586,22 +13589,22 @@
       <c r="A206" s="2">
         <v>2025</v>
       </c>
-      <c r="B206" s="71" t="s">
+      <c r="B206" s="53" t="s">
         <v>970</v>
       </c>
-      <c r="C206" s="71" t="s">
+      <c r="C206" s="53" t="s">
         <v>971</v>
       </c>
-      <c r="D206" s="71" t="s">
+      <c r="D206" s="53" t="s">
         <v>950</v>
       </c>
-      <c r="E206" s="71" t="s">
+      <c r="E206" s="53" t="s">
         <v>766</v>
       </c>
-      <c r="F206" s="71" t="s">
+      <c r="F206" s="53" t="s">
         <v>972</v>
       </c>
-      <c r="G206" s="71" t="s">
+      <c r="G206" s="53" t="s">
         <v>965</v>
       </c>
       <c r="H206" s="2" t="s">
@@ -13612,22 +13615,22 @@
       <c r="A207" s="2">
         <v>2025</v>
       </c>
-      <c r="B207" s="72" t="s">
+      <c r="B207" s="54" t="s">
         <v>932</v>
       </c>
-      <c r="C207" s="72" t="s">
+      <c r="C207" s="54" t="s">
         <v>973</v>
       </c>
-      <c r="D207" s="72" t="s">
+      <c r="D207" s="54" t="s">
         <v>951</v>
       </c>
-      <c r="E207" s="72" t="s">
+      <c r="E207" s="54" t="s">
         <v>241</v>
       </c>
-      <c r="F207" s="72" t="s">
+      <c r="F207" s="54" t="s">
         <v>302</v>
       </c>
-      <c r="G207" s="72" t="s">
+      <c r="G207" s="54" t="s">
         <v>766</v>
       </c>
       <c r="H207" s="2" t="s">
@@ -13638,22 +13641,22 @@
       <c r="A208" s="2">
         <v>2025</v>
       </c>
-      <c r="B208" s="71" t="s">
+      <c r="B208" s="53" t="s">
         <v>933</v>
       </c>
-      <c r="C208" s="71" t="s">
+      <c r="C208" s="53" t="s">
         <v>934</v>
       </c>
-      <c r="D208" s="71" t="s">
+      <c r="D208" s="53" t="s">
         <v>952</v>
       </c>
-      <c r="E208" s="71" t="s">
+      <c r="E208" s="53" t="s">
         <v>182</v>
       </c>
-      <c r="F208" s="71" t="s">
+      <c r="F208" s="53" t="s">
         <v>205</v>
       </c>
-      <c r="G208" s="71" t="s">
+      <c r="G208" s="53" t="s">
         <v>37</v>
       </c>
       <c r="H208" s="2" t="s">
@@ -13664,22 +13667,22 @@
       <c r="A209" s="2">
         <v>2025</v>
       </c>
-      <c r="B209" s="72" t="s">
+      <c r="B209" s="54" t="s">
         <v>935</v>
       </c>
-      <c r="C209" s="72" t="s">
+      <c r="C209" s="54" t="s">
         <v>936</v>
       </c>
-      <c r="D209" s="72" t="s">
+      <c r="D209" s="54" t="s">
         <v>953</v>
       </c>
-      <c r="E209" s="72" t="s">
+      <c r="E209" s="54" t="s">
         <v>974</v>
       </c>
-      <c r="F209" s="72" t="s">
+      <c r="F209" s="54" t="s">
         <v>291</v>
       </c>
-      <c r="G209" s="72" t="s">
+      <c r="G209" s="54" t="s">
         <v>39</v>
       </c>
       <c r="H209" s="2" t="s">
@@ -13690,22 +13693,22 @@
       <c r="A210" s="2">
         <v>2025</v>
       </c>
-      <c r="B210" s="71" t="s">
+      <c r="B210" s="53" t="s">
         <v>975</v>
       </c>
-      <c r="C210" s="71" t="s">
+      <c r="C210" s="53" t="s">
         <v>937</v>
       </c>
-      <c r="D210" s="71" t="s">
+      <c r="D210" s="53" t="s">
         <v>954</v>
       </c>
-      <c r="E210" s="71" t="s">
+      <c r="E210" s="53" t="s">
         <v>241</v>
       </c>
-      <c r="F210" s="71" t="s">
+      <c r="F210" s="53" t="s">
         <v>766</v>
       </c>
-      <c r="G210" s="71" t="s">
+      <c r="G210" s="53" t="s">
         <v>966</v>
       </c>
       <c r="H210" s="2" t="s">
@@ -13716,22 +13719,22 @@
       <c r="A211" s="2">
         <v>2025</v>
       </c>
-      <c r="B211" s="72" t="s">
+      <c r="B211" s="54" t="s">
         <v>976</v>
       </c>
-      <c r="C211" s="72" t="s">
+      <c r="C211" s="54" t="s">
         <v>977</v>
       </c>
-      <c r="D211" s="72" t="s">
+      <c r="D211" s="54" t="s">
         <v>955</v>
       </c>
-      <c r="E211" s="72" t="s">
+      <c r="E211" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="F211" s="72" t="s">
+      <c r="F211" s="54" t="s">
         <v>302</v>
       </c>
-      <c r="G211" s="72" t="s">
+      <c r="G211" s="54" t="s">
         <v>978</v>
       </c>
       <c r="H211" s="2" t="s">
@@ -13742,22 +13745,22 @@
       <c r="A212" s="2">
         <v>2025</v>
       </c>
-      <c r="B212" s="71" t="s">
+      <c r="B212" s="53" t="s">
         <v>257</v>
       </c>
-      <c r="C212" s="71" t="s">
+      <c r="C212" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="D212" s="71" t="s">
+      <c r="D212" s="53" t="s">
         <v>956</v>
       </c>
-      <c r="E212" s="71" t="s">
+      <c r="E212" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="F212" s="71" t="s">
+      <c r="F212" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="G212" s="71" t="s">
+      <c r="G212" s="53" t="s">
         <v>979</v>
       </c>
       <c r="H212" s="2" t="s">
@@ -13768,22 +13771,22 @@
       <c r="A213" s="2">
         <v>2025</v>
       </c>
-      <c r="B213" s="72" t="s">
+      <c r="B213" s="54" t="s">
         <v>938</v>
       </c>
-      <c r="C213" s="72" t="s">
+      <c r="C213" s="54" t="s">
         <v>218</v>
       </c>
-      <c r="D213" s="72" t="s">
+      <c r="D213" s="54" t="s">
         <v>957</v>
       </c>
-      <c r="E213" s="72" t="s">
+      <c r="E213" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F213" s="72" t="s">
+      <c r="F213" s="54" t="s">
         <v>583</v>
       </c>
-      <c r="G213" s="72" t="s">
+      <c r="G213" s="54" t="s">
         <v>980</v>
       </c>
       <c r="H213" s="2" t="s">
@@ -13794,1503 +13797,1503 @@
       <c r="A214" s="2">
         <v>2025</v>
       </c>
-      <c r="B214" s="71" t="s">
+      <c r="B214" s="53" t="s">
         <v>939</v>
       </c>
-      <c r="C214" s="71" t="s">
+      <c r="C214" s="53" t="s">
         <v>934</v>
       </c>
-      <c r="D214" s="71" t="s">
+      <c r="D214" s="53" t="s">
         <v>958</v>
       </c>
-      <c r="E214" s="71" t="s">
+      <c r="E214" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="F214" s="71" t="s">
+      <c r="F214" s="53" t="s">
         <v>959</v>
       </c>
-      <c r="G214" s="71" t="s">
+      <c r="G214" s="53" t="s">
         <v>981</v>
       </c>
       <c r="H214" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="215" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A215" s="73">
+    <row r="215" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A215" s="55">
         <v>2026</v>
       </c>
-      <c r="B215" s="73" t="s">
+      <c r="B215" s="55" t="s">
         <v>982</v>
       </c>
-      <c r="C215" s="73" t="s">
+      <c r="C215" s="55" t="s">
         <v>442</v>
       </c>
-      <c r="E215" s="73" t="s">
+      <c r="E215" s="55" t="s">
         <v>241</v>
       </c>
-      <c r="F215" s="73" t="s">
+      <c r="F215" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="K215" s="74"/>
-      <c r="L215" s="74"/>
-      <c r="M215" s="74"/>
-      <c r="N215" s="74"/>
-      <c r="O215" s="74"/>
-      <c r="P215" s="74"/>
-      <c r="Q215" s="74"/>
-      <c r="R215" s="74"/>
-      <c r="S215" s="74"/>
-      <c r="T215" s="74"/>
-      <c r="U215" s="74"/>
-      <c r="V215" s="74"/>
-      <c r="W215" s="74"/>
-      <c r="X215" s="74"/>
-      <c r="Y215" s="74"/>
-      <c r="Z215" s="74"/>
-      <c r="AA215" s="74"/>
-      <c r="AB215" s="74"/>
-      <c r="AC215" s="74"/>
-      <c r="AD215" s="74"/>
-      <c r="AE215" s="74"/>
-      <c r="AF215" s="74"/>
-      <c r="AG215" s="74"/>
-      <c r="AH215" s="74"/>
-      <c r="AI215" s="74"/>
-      <c r="AJ215" s="74"/>
-      <c r="AK215" s="74"/>
-      <c r="AL215" s="74"/>
-      <c r="AM215" s="74"/>
-      <c r="AN215" s="74"/>
-      <c r="AO215" s="74"/>
-      <c r="AP215" s="74"/>
-      <c r="AQ215" s="74"/>
-      <c r="AR215" s="74"/>
-      <c r="AS215" s="74"/>
-      <c r="AT215" s="74"/>
-      <c r="AU215" s="74"/>
-      <c r="AV215" s="74"/>
-      <c r="AW215" s="74"/>
-      <c r="AX215" s="74"/>
-      <c r="AY215" s="74"/>
-      <c r="AZ215" s="74"/>
-      <c r="BA215" s="74"/>
-      <c r="BB215" s="74"/>
-      <c r="BC215" s="74"/>
-      <c r="BD215" s="74"/>
-      <c r="BE215" s="74"/>
-      <c r="BF215" s="74"/>
-      <c r="BG215" s="74"/>
-      <c r="BH215" s="74"/>
-      <c r="BI215" s="74"/>
-      <c r="BJ215" s="74"/>
-      <c r="BK215" s="74"/>
-      <c r="BL215" s="74"/>
-      <c r="BM215" s="74"/>
-      <c r="BN215" s="74"/>
-      <c r="BO215" s="74"/>
-      <c r="BP215" s="74"/>
-      <c r="BQ215" s="74"/>
-      <c r="BR215" s="74"/>
-      <c r="BS215" s="74"/>
-      <c r="BT215" s="74"/>
-      <c r="BU215" s="74"/>
-      <c r="BV215" s="74"/>
-      <c r="BW215" s="74"/>
-      <c r="BX215" s="74"/>
-      <c r="BY215" s="74"/>
-      <c r="BZ215" s="74"/>
-      <c r="CA215" s="74"/>
-      <c r="CB215" s="74"/>
-      <c r="CC215" s="74"/>
-      <c r="CD215" s="74"/>
-      <c r="CE215" s="74"/>
-      <c r="CF215" s="74"/>
-      <c r="CG215" s="74"/>
-      <c r="CH215" s="74"/>
-      <c r="CI215" s="74"/>
-      <c r="CJ215" s="74"/>
-      <c r="CK215" s="74"/>
-      <c r="CL215" s="74"/>
-      <c r="CM215" s="74"/>
-      <c r="CN215" s="74"/>
-      <c r="CO215" s="74"/>
-      <c r="CP215" s="74"/>
-      <c r="CQ215" s="74"/>
-      <c r="CR215" s="74"/>
-      <c r="CS215" s="74"/>
-      <c r="CT215" s="74"/>
-      <c r="CU215" s="74"/>
-      <c r="CV215" s="74"/>
-      <c r="CW215" s="74"/>
-      <c r="CX215" s="74"/>
-      <c r="CY215" s="74"/>
-      <c r="CZ215" s="74"/>
-      <c r="DA215" s="74"/>
-      <c r="DB215" s="74"/>
-      <c r="DC215" s="74"/>
-      <c r="DD215" s="74"/>
-      <c r="DE215" s="74"/>
-      <c r="DF215" s="74"/>
-      <c r="DG215" s="74"/>
-      <c r="DH215" s="74"/>
-      <c r="DI215" s="74"/>
-      <c r="DJ215" s="74"/>
-      <c r="DK215" s="74"/>
-      <c r="DL215" s="74"/>
-      <c r="DM215" s="74"/>
-    </row>
-    <row r="216" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A216" s="73">
+      <c r="K215" s="56"/>
+      <c r="L215" s="56"/>
+      <c r="M215" s="56"/>
+      <c r="N215" s="56"/>
+      <c r="O215" s="56"/>
+      <c r="P215" s="56"/>
+      <c r="Q215" s="56"/>
+      <c r="R215" s="56"/>
+      <c r="S215" s="56"/>
+      <c r="T215" s="56"/>
+      <c r="U215" s="56"/>
+      <c r="V215" s="56"/>
+      <c r="W215" s="56"/>
+      <c r="X215" s="56"/>
+      <c r="Y215" s="56"/>
+      <c r="Z215" s="56"/>
+      <c r="AA215" s="56"/>
+      <c r="AB215" s="56"/>
+      <c r="AC215" s="56"/>
+      <c r="AD215" s="56"/>
+      <c r="AE215" s="56"/>
+      <c r="AF215" s="56"/>
+      <c r="AG215" s="56"/>
+      <c r="AH215" s="56"/>
+      <c r="AI215" s="56"/>
+      <c r="AJ215" s="56"/>
+      <c r="AK215" s="56"/>
+      <c r="AL215" s="56"/>
+      <c r="AM215" s="56"/>
+      <c r="AN215" s="56"/>
+      <c r="AO215" s="56"/>
+      <c r="AP215" s="56"/>
+      <c r="AQ215" s="56"/>
+      <c r="AR215" s="56"/>
+      <c r="AS215" s="56"/>
+      <c r="AT215" s="56"/>
+      <c r="AU215" s="56"/>
+      <c r="AV215" s="56"/>
+      <c r="AW215" s="56"/>
+      <c r="AX215" s="56"/>
+      <c r="AY215" s="56"/>
+      <c r="AZ215" s="56"/>
+      <c r="BA215" s="56"/>
+      <c r="BB215" s="56"/>
+      <c r="BC215" s="56"/>
+      <c r="BD215" s="56"/>
+      <c r="BE215" s="56"/>
+      <c r="BF215" s="56"/>
+      <c r="BG215" s="56"/>
+      <c r="BH215" s="56"/>
+      <c r="BI215" s="56"/>
+      <c r="BJ215" s="56"/>
+      <c r="BK215" s="56"/>
+      <c r="BL215" s="56"/>
+      <c r="BM215" s="56"/>
+      <c r="BN215" s="56"/>
+      <c r="BO215" s="56"/>
+      <c r="BP215" s="56"/>
+      <c r="BQ215" s="56"/>
+      <c r="BR215" s="56"/>
+      <c r="BS215" s="56"/>
+      <c r="BT215" s="56"/>
+      <c r="BU215" s="56"/>
+      <c r="BV215" s="56"/>
+      <c r="BW215" s="56"/>
+      <c r="BX215" s="56"/>
+      <c r="BY215" s="56"/>
+      <c r="BZ215" s="56"/>
+      <c r="CA215" s="56"/>
+      <c r="CB215" s="56"/>
+      <c r="CC215" s="56"/>
+      <c r="CD215" s="56"/>
+      <c r="CE215" s="56"/>
+      <c r="CF215" s="56"/>
+      <c r="CG215" s="56"/>
+      <c r="CH215" s="56"/>
+      <c r="CI215" s="56"/>
+      <c r="CJ215" s="56"/>
+      <c r="CK215" s="56"/>
+      <c r="CL215" s="56"/>
+      <c r="CM215" s="56"/>
+      <c r="CN215" s="56"/>
+      <c r="CO215" s="56"/>
+      <c r="CP215" s="56"/>
+      <c r="CQ215" s="56"/>
+      <c r="CR215" s="56"/>
+      <c r="CS215" s="56"/>
+      <c r="CT215" s="56"/>
+      <c r="CU215" s="56"/>
+      <c r="CV215" s="56"/>
+      <c r="CW215" s="56"/>
+      <c r="CX215" s="56"/>
+      <c r="CY215" s="56"/>
+      <c r="CZ215" s="56"/>
+      <c r="DA215" s="56"/>
+      <c r="DB215" s="56"/>
+      <c r="DC215" s="56"/>
+      <c r="DD215" s="56"/>
+      <c r="DE215" s="56"/>
+      <c r="DF215" s="56"/>
+      <c r="DG215" s="56"/>
+      <c r="DH215" s="56"/>
+      <c r="DI215" s="56"/>
+      <c r="DJ215" s="56"/>
+      <c r="DK215" s="56"/>
+      <c r="DL215" s="56"/>
+      <c r="DM215" s="56"/>
+    </row>
+    <row r="216" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A216" s="55">
         <v>2026</v>
       </c>
-      <c r="B216" s="73" t="s">
+      <c r="B216" s="55" t="s">
         <v>983</v>
       </c>
-      <c r="C216" s="73" t="s">
+      <c r="C216" s="55" t="s">
         <v>984</v>
       </c>
-      <c r="E216" s="73" t="s">
+      <c r="E216" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="F216" s="73" t="s">
+      <c r="F216" s="55" t="s">
         <v>583</v>
       </c>
-      <c r="K216" s="74"/>
-      <c r="L216" s="74"/>
-      <c r="M216" s="74"/>
-      <c r="N216" s="74"/>
-      <c r="O216" s="74"/>
-      <c r="P216" s="74"/>
-      <c r="Q216" s="74"/>
-      <c r="R216" s="74"/>
-      <c r="S216" s="74"/>
-      <c r="T216" s="74"/>
-      <c r="U216" s="74"/>
-      <c r="V216" s="74"/>
-      <c r="W216" s="74"/>
-      <c r="X216" s="74"/>
-      <c r="Y216" s="74"/>
-      <c r="Z216" s="74"/>
-      <c r="AA216" s="74"/>
-      <c r="AB216" s="74"/>
-      <c r="AC216" s="74"/>
-      <c r="AD216" s="74"/>
-      <c r="AE216" s="74"/>
-      <c r="AF216" s="74"/>
-      <c r="AG216" s="74"/>
-      <c r="AH216" s="74"/>
-      <c r="AI216" s="74"/>
-      <c r="AJ216" s="74"/>
-      <c r="AK216" s="74"/>
-      <c r="AL216" s="74"/>
-      <c r="AM216" s="74"/>
-      <c r="AN216" s="74"/>
-      <c r="AO216" s="74"/>
-      <c r="AP216" s="74"/>
-      <c r="AQ216" s="74"/>
-      <c r="AR216" s="74"/>
-      <c r="AS216" s="74"/>
-      <c r="AT216" s="74"/>
-      <c r="AU216" s="74"/>
-      <c r="AV216" s="74"/>
-      <c r="AW216" s="74"/>
-      <c r="AX216" s="74"/>
-      <c r="AY216" s="74"/>
-      <c r="AZ216" s="74"/>
-      <c r="BA216" s="74"/>
-      <c r="BB216" s="74"/>
-      <c r="BC216" s="74"/>
-      <c r="BD216" s="74"/>
-      <c r="BE216" s="74"/>
-      <c r="BF216" s="74"/>
-      <c r="BG216" s="74"/>
-      <c r="BH216" s="74"/>
-      <c r="BI216" s="74"/>
-      <c r="BJ216" s="74"/>
-      <c r="BK216" s="74"/>
-      <c r="BL216" s="74"/>
-      <c r="BM216" s="74"/>
-      <c r="BN216" s="74"/>
-      <c r="BO216" s="74"/>
-      <c r="BP216" s="74"/>
-      <c r="BQ216" s="74"/>
-      <c r="BR216" s="74"/>
-      <c r="BS216" s="74"/>
-      <c r="BT216" s="74"/>
-      <c r="BU216" s="74"/>
-      <c r="BV216" s="74"/>
-      <c r="BW216" s="74"/>
-      <c r="BX216" s="74"/>
-      <c r="BY216" s="74"/>
-      <c r="BZ216" s="74"/>
-      <c r="CA216" s="74"/>
-      <c r="CB216" s="74"/>
-      <c r="CC216" s="74"/>
-      <c r="CD216" s="74"/>
-      <c r="CE216" s="74"/>
-      <c r="CF216" s="74"/>
-      <c r="CG216" s="74"/>
-      <c r="CH216" s="74"/>
-      <c r="CI216" s="74"/>
-      <c r="CJ216" s="74"/>
-      <c r="CK216" s="74"/>
-      <c r="CL216" s="74"/>
-      <c r="CM216" s="74"/>
-      <c r="CN216" s="74"/>
-      <c r="CO216" s="74"/>
-      <c r="CP216" s="74"/>
-      <c r="CQ216" s="74"/>
-      <c r="CR216" s="74"/>
-      <c r="CS216" s="74"/>
-      <c r="CT216" s="74"/>
-      <c r="CU216" s="74"/>
-      <c r="CV216" s="74"/>
-      <c r="CW216" s="74"/>
-      <c r="CX216" s="74"/>
-      <c r="CY216" s="74"/>
-      <c r="CZ216" s="74"/>
-      <c r="DA216" s="74"/>
-      <c r="DB216" s="74"/>
-      <c r="DC216" s="74"/>
-      <c r="DD216" s="74"/>
-      <c r="DE216" s="74"/>
-      <c r="DF216" s="74"/>
-      <c r="DG216" s="74"/>
-      <c r="DH216" s="74"/>
-      <c r="DI216" s="74"/>
-      <c r="DJ216" s="74"/>
-      <c r="DK216" s="74"/>
-      <c r="DL216" s="74"/>
-      <c r="DM216" s="74"/>
-    </row>
-    <row r="217" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A217" s="73">
+      <c r="K216" s="56"/>
+      <c r="L216" s="56"/>
+      <c r="M216" s="56"/>
+      <c r="N216" s="56"/>
+      <c r="O216" s="56"/>
+      <c r="P216" s="56"/>
+      <c r="Q216" s="56"/>
+      <c r="R216" s="56"/>
+      <c r="S216" s="56"/>
+      <c r="T216" s="56"/>
+      <c r="U216" s="56"/>
+      <c r="V216" s="56"/>
+      <c r="W216" s="56"/>
+      <c r="X216" s="56"/>
+      <c r="Y216" s="56"/>
+      <c r="Z216" s="56"/>
+      <c r="AA216" s="56"/>
+      <c r="AB216" s="56"/>
+      <c r="AC216" s="56"/>
+      <c r="AD216" s="56"/>
+      <c r="AE216" s="56"/>
+      <c r="AF216" s="56"/>
+      <c r="AG216" s="56"/>
+      <c r="AH216" s="56"/>
+      <c r="AI216" s="56"/>
+      <c r="AJ216" s="56"/>
+      <c r="AK216" s="56"/>
+      <c r="AL216" s="56"/>
+      <c r="AM216" s="56"/>
+      <c r="AN216" s="56"/>
+      <c r="AO216" s="56"/>
+      <c r="AP216" s="56"/>
+      <c r="AQ216" s="56"/>
+      <c r="AR216" s="56"/>
+      <c r="AS216" s="56"/>
+      <c r="AT216" s="56"/>
+      <c r="AU216" s="56"/>
+      <c r="AV216" s="56"/>
+      <c r="AW216" s="56"/>
+      <c r="AX216" s="56"/>
+      <c r="AY216" s="56"/>
+      <c r="AZ216" s="56"/>
+      <c r="BA216" s="56"/>
+      <c r="BB216" s="56"/>
+      <c r="BC216" s="56"/>
+      <c r="BD216" s="56"/>
+      <c r="BE216" s="56"/>
+      <c r="BF216" s="56"/>
+      <c r="BG216" s="56"/>
+      <c r="BH216" s="56"/>
+      <c r="BI216" s="56"/>
+      <c r="BJ216" s="56"/>
+      <c r="BK216" s="56"/>
+      <c r="BL216" s="56"/>
+      <c r="BM216" s="56"/>
+      <c r="BN216" s="56"/>
+      <c r="BO216" s="56"/>
+      <c r="BP216" s="56"/>
+      <c r="BQ216" s="56"/>
+      <c r="BR216" s="56"/>
+      <c r="BS216" s="56"/>
+      <c r="BT216" s="56"/>
+      <c r="BU216" s="56"/>
+      <c r="BV216" s="56"/>
+      <c r="BW216" s="56"/>
+      <c r="BX216" s="56"/>
+      <c r="BY216" s="56"/>
+      <c r="BZ216" s="56"/>
+      <c r="CA216" s="56"/>
+      <c r="CB216" s="56"/>
+      <c r="CC216" s="56"/>
+      <c r="CD216" s="56"/>
+      <c r="CE216" s="56"/>
+      <c r="CF216" s="56"/>
+      <c r="CG216" s="56"/>
+      <c r="CH216" s="56"/>
+      <c r="CI216" s="56"/>
+      <c r="CJ216" s="56"/>
+      <c r="CK216" s="56"/>
+      <c r="CL216" s="56"/>
+      <c r="CM216" s="56"/>
+      <c r="CN216" s="56"/>
+      <c r="CO216" s="56"/>
+      <c r="CP216" s="56"/>
+      <c r="CQ216" s="56"/>
+      <c r="CR216" s="56"/>
+      <c r="CS216" s="56"/>
+      <c r="CT216" s="56"/>
+      <c r="CU216" s="56"/>
+      <c r="CV216" s="56"/>
+      <c r="CW216" s="56"/>
+      <c r="CX216" s="56"/>
+      <c r="CY216" s="56"/>
+      <c r="CZ216" s="56"/>
+      <c r="DA216" s="56"/>
+      <c r="DB216" s="56"/>
+      <c r="DC216" s="56"/>
+      <c r="DD216" s="56"/>
+      <c r="DE216" s="56"/>
+      <c r="DF216" s="56"/>
+      <c r="DG216" s="56"/>
+      <c r="DH216" s="56"/>
+      <c r="DI216" s="56"/>
+      <c r="DJ216" s="56"/>
+      <c r="DK216" s="56"/>
+      <c r="DL216" s="56"/>
+      <c r="DM216" s="56"/>
+    </row>
+    <row r="217" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A217" s="55">
         <v>2026</v>
       </c>
-      <c r="B217" s="73" t="s">
+      <c r="B217" s="55" t="s">
         <v>985</v>
       </c>
-      <c r="C217" s="73" t="s">
+      <c r="C217" s="55" t="s">
         <v>680</v>
       </c>
-      <c r="E217" s="75" t="s">
+      <c r="E217" s="57" t="s">
         <v>464</v>
       </c>
-      <c r="F217" s="73" t="s">
+      <c r="F217" s="55" t="s">
         <v>472</v>
       </c>
-      <c r="K217" s="74"/>
-      <c r="L217" s="74"/>
-      <c r="M217" s="74"/>
-      <c r="N217" s="74"/>
-      <c r="O217" s="74"/>
-      <c r="P217" s="74"/>
-      <c r="Q217" s="74"/>
-      <c r="R217" s="74"/>
-      <c r="S217" s="74"/>
-      <c r="T217" s="74"/>
-      <c r="U217" s="74"/>
-      <c r="V217" s="74"/>
-      <c r="W217" s="74"/>
-      <c r="X217" s="74"/>
-      <c r="Y217" s="74"/>
-      <c r="Z217" s="74"/>
-      <c r="AA217" s="74"/>
-      <c r="AB217" s="74"/>
-      <c r="AC217" s="74"/>
-      <c r="AD217" s="74"/>
-      <c r="AE217" s="74"/>
-      <c r="AF217" s="74"/>
-      <c r="AG217" s="74"/>
-      <c r="AH217" s="74"/>
-      <c r="AI217" s="74"/>
-      <c r="AJ217" s="74"/>
-      <c r="AK217" s="74"/>
-      <c r="AL217" s="74"/>
-      <c r="AM217" s="74"/>
-      <c r="AN217" s="74"/>
-      <c r="AO217" s="74"/>
-      <c r="AP217" s="74"/>
-      <c r="AQ217" s="74"/>
-      <c r="AR217" s="74"/>
-      <c r="AS217" s="74"/>
-      <c r="AT217" s="74"/>
-      <c r="AU217" s="74"/>
-      <c r="AV217" s="74"/>
-      <c r="AW217" s="74"/>
-      <c r="AX217" s="74"/>
-      <c r="AY217" s="74"/>
-      <c r="AZ217" s="74"/>
-      <c r="BA217" s="74"/>
-      <c r="BB217" s="74"/>
-      <c r="BC217" s="74"/>
-      <c r="BD217" s="74"/>
-      <c r="BE217" s="74"/>
-      <c r="BF217" s="74"/>
-      <c r="BG217" s="74"/>
-      <c r="BH217" s="74"/>
-      <c r="BI217" s="74"/>
-      <c r="BJ217" s="74"/>
-      <c r="BK217" s="74"/>
-      <c r="BL217" s="74"/>
-      <c r="BM217" s="74"/>
-      <c r="BN217" s="74"/>
-      <c r="BO217" s="74"/>
-      <c r="BP217" s="74"/>
-      <c r="BQ217" s="74"/>
-      <c r="BR217" s="74"/>
-      <c r="BS217" s="74"/>
-      <c r="BT217" s="74"/>
-      <c r="BU217" s="74"/>
-      <c r="BV217" s="74"/>
-      <c r="BW217" s="74"/>
-      <c r="BX217" s="74"/>
-      <c r="BY217" s="74"/>
-      <c r="BZ217" s="74"/>
-      <c r="CA217" s="74"/>
-      <c r="CB217" s="74"/>
-      <c r="CC217" s="74"/>
-      <c r="CD217" s="74"/>
-      <c r="CE217" s="74"/>
-      <c r="CF217" s="74"/>
-      <c r="CG217" s="74"/>
-      <c r="CH217" s="74"/>
-      <c r="CI217" s="74"/>
-      <c r="CJ217" s="74"/>
-      <c r="CK217" s="74"/>
-      <c r="CL217" s="74"/>
-      <c r="CM217" s="74"/>
-      <c r="CN217" s="74"/>
-      <c r="CO217" s="74"/>
-      <c r="CP217" s="74"/>
-      <c r="CQ217" s="74"/>
-      <c r="CR217" s="74"/>
-      <c r="CS217" s="74"/>
-      <c r="CT217" s="74"/>
-      <c r="CU217" s="74"/>
-      <c r="CV217" s="74"/>
-      <c r="CW217" s="74"/>
-      <c r="CX217" s="74"/>
-      <c r="CY217" s="74"/>
-      <c r="CZ217" s="74"/>
-      <c r="DA217" s="74"/>
-      <c r="DB217" s="74"/>
-      <c r="DC217" s="74"/>
-      <c r="DD217" s="74"/>
-      <c r="DE217" s="74"/>
-      <c r="DF217" s="74"/>
-      <c r="DG217" s="74"/>
-      <c r="DH217" s="74"/>
-      <c r="DI217" s="74"/>
-      <c r="DJ217" s="74"/>
-      <c r="DK217" s="74"/>
-      <c r="DL217" s="74"/>
-      <c r="DM217" s="74"/>
-    </row>
-    <row r="218" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A218" s="73">
+      <c r="K217" s="56"/>
+      <c r="L217" s="56"/>
+      <c r="M217" s="56"/>
+      <c r="N217" s="56"/>
+      <c r="O217" s="56"/>
+      <c r="P217" s="56"/>
+      <c r="Q217" s="56"/>
+      <c r="R217" s="56"/>
+      <c r="S217" s="56"/>
+      <c r="T217" s="56"/>
+      <c r="U217" s="56"/>
+      <c r="V217" s="56"/>
+      <c r="W217" s="56"/>
+      <c r="X217" s="56"/>
+      <c r="Y217" s="56"/>
+      <c r="Z217" s="56"/>
+      <c r="AA217" s="56"/>
+      <c r="AB217" s="56"/>
+      <c r="AC217" s="56"/>
+      <c r="AD217" s="56"/>
+      <c r="AE217" s="56"/>
+      <c r="AF217" s="56"/>
+      <c r="AG217" s="56"/>
+      <c r="AH217" s="56"/>
+      <c r="AI217" s="56"/>
+      <c r="AJ217" s="56"/>
+      <c r="AK217" s="56"/>
+      <c r="AL217" s="56"/>
+      <c r="AM217" s="56"/>
+      <c r="AN217" s="56"/>
+      <c r="AO217" s="56"/>
+      <c r="AP217" s="56"/>
+      <c r="AQ217" s="56"/>
+      <c r="AR217" s="56"/>
+      <c r="AS217" s="56"/>
+      <c r="AT217" s="56"/>
+      <c r="AU217" s="56"/>
+      <c r="AV217" s="56"/>
+      <c r="AW217" s="56"/>
+      <c r="AX217" s="56"/>
+      <c r="AY217" s="56"/>
+      <c r="AZ217" s="56"/>
+      <c r="BA217" s="56"/>
+      <c r="BB217" s="56"/>
+      <c r="BC217" s="56"/>
+      <c r="BD217" s="56"/>
+      <c r="BE217" s="56"/>
+      <c r="BF217" s="56"/>
+      <c r="BG217" s="56"/>
+      <c r="BH217" s="56"/>
+      <c r="BI217" s="56"/>
+      <c r="BJ217" s="56"/>
+      <c r="BK217" s="56"/>
+      <c r="BL217" s="56"/>
+      <c r="BM217" s="56"/>
+      <c r="BN217" s="56"/>
+      <c r="BO217" s="56"/>
+      <c r="BP217" s="56"/>
+      <c r="BQ217" s="56"/>
+      <c r="BR217" s="56"/>
+      <c r="BS217" s="56"/>
+      <c r="BT217" s="56"/>
+      <c r="BU217" s="56"/>
+      <c r="BV217" s="56"/>
+      <c r="BW217" s="56"/>
+      <c r="BX217" s="56"/>
+      <c r="BY217" s="56"/>
+      <c r="BZ217" s="56"/>
+      <c r="CA217" s="56"/>
+      <c r="CB217" s="56"/>
+      <c r="CC217" s="56"/>
+      <c r="CD217" s="56"/>
+      <c r="CE217" s="56"/>
+      <c r="CF217" s="56"/>
+      <c r="CG217" s="56"/>
+      <c r="CH217" s="56"/>
+      <c r="CI217" s="56"/>
+      <c r="CJ217" s="56"/>
+      <c r="CK217" s="56"/>
+      <c r="CL217" s="56"/>
+      <c r="CM217" s="56"/>
+      <c r="CN217" s="56"/>
+      <c r="CO217" s="56"/>
+      <c r="CP217" s="56"/>
+      <c r="CQ217" s="56"/>
+      <c r="CR217" s="56"/>
+      <c r="CS217" s="56"/>
+      <c r="CT217" s="56"/>
+      <c r="CU217" s="56"/>
+      <c r="CV217" s="56"/>
+      <c r="CW217" s="56"/>
+      <c r="CX217" s="56"/>
+      <c r="CY217" s="56"/>
+      <c r="CZ217" s="56"/>
+      <c r="DA217" s="56"/>
+      <c r="DB217" s="56"/>
+      <c r="DC217" s="56"/>
+      <c r="DD217" s="56"/>
+      <c r="DE217" s="56"/>
+      <c r="DF217" s="56"/>
+      <c r="DG217" s="56"/>
+      <c r="DH217" s="56"/>
+      <c r="DI217" s="56"/>
+      <c r="DJ217" s="56"/>
+      <c r="DK217" s="56"/>
+      <c r="DL217" s="56"/>
+      <c r="DM217" s="56"/>
+    </row>
+    <row r="218" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A218" s="55">
         <v>2026</v>
       </c>
-      <c r="B218" s="73" t="s">
+      <c r="B218" s="55" t="s">
         <v>986</v>
       </c>
-      <c r="C218" s="73" t="s">
+      <c r="C218" s="55" t="s">
         <v>987</v>
       </c>
-      <c r="E218" s="73" t="s">
+      <c r="E218" s="55" t="s">
         <v>182</v>
       </c>
-      <c r="F218" s="73" t="s">
+      <c r="F218" s="55" t="s">
         <v>988</v>
       </c>
-      <c r="K218" s="74"/>
-      <c r="L218" s="74"/>
-      <c r="M218" s="74"/>
-      <c r="N218" s="74"/>
-      <c r="O218" s="74"/>
-      <c r="P218" s="74"/>
-      <c r="Q218" s="74"/>
-      <c r="R218" s="74"/>
-      <c r="S218" s="74"/>
-      <c r="T218" s="74"/>
-      <c r="U218" s="74"/>
-      <c r="V218" s="74"/>
-      <c r="W218" s="74"/>
-      <c r="X218" s="74"/>
-      <c r="Y218" s="74"/>
-      <c r="Z218" s="74"/>
-      <c r="AA218" s="74"/>
-      <c r="AB218" s="74"/>
-      <c r="AC218" s="74"/>
-      <c r="AD218" s="74"/>
-      <c r="AE218" s="74"/>
-      <c r="AF218" s="74"/>
-      <c r="AG218" s="74"/>
-      <c r="AH218" s="74"/>
-      <c r="AI218" s="74"/>
-      <c r="AJ218" s="74"/>
-      <c r="AK218" s="74"/>
-      <c r="AL218" s="74"/>
-      <c r="AM218" s="74"/>
-      <c r="AN218" s="74"/>
-      <c r="AO218" s="74"/>
-      <c r="AP218" s="74"/>
-      <c r="AQ218" s="74"/>
-      <c r="AR218" s="74"/>
-      <c r="AS218" s="74"/>
-      <c r="AT218" s="74"/>
-      <c r="AU218" s="74"/>
-      <c r="AV218" s="74"/>
-      <c r="AW218" s="74"/>
-      <c r="AX218" s="74"/>
-      <c r="AY218" s="74"/>
-      <c r="AZ218" s="74"/>
-      <c r="BA218" s="74"/>
-      <c r="BB218" s="74"/>
-      <c r="BC218" s="74"/>
-      <c r="BD218" s="74"/>
-      <c r="BE218" s="74"/>
-      <c r="BF218" s="74"/>
-      <c r="BG218" s="74"/>
-      <c r="BH218" s="74"/>
-      <c r="BI218" s="74"/>
-      <c r="BJ218" s="74"/>
-      <c r="BK218" s="74"/>
-      <c r="BL218" s="74"/>
-      <c r="BM218" s="74"/>
-      <c r="BN218" s="74"/>
-      <c r="BO218" s="74"/>
-      <c r="BP218" s="74"/>
-      <c r="BQ218" s="74"/>
-      <c r="BR218" s="74"/>
-      <c r="BS218" s="74"/>
-      <c r="BT218" s="74"/>
-      <c r="BU218" s="74"/>
-      <c r="BV218" s="74"/>
-      <c r="BW218" s="74"/>
-      <c r="BX218" s="74"/>
-      <c r="BY218" s="74"/>
-      <c r="BZ218" s="74"/>
-      <c r="CA218" s="74"/>
-      <c r="CB218" s="74"/>
-      <c r="CC218" s="74"/>
-      <c r="CD218" s="74"/>
-      <c r="CE218" s="74"/>
-      <c r="CF218" s="74"/>
-      <c r="CG218" s="74"/>
-      <c r="CH218" s="74"/>
-      <c r="CI218" s="74"/>
-      <c r="CJ218" s="74"/>
-      <c r="CK218" s="74"/>
-      <c r="CL218" s="74"/>
-      <c r="CM218" s="74"/>
-      <c r="CN218" s="74"/>
-      <c r="CO218" s="74"/>
-      <c r="CP218" s="74"/>
-      <c r="CQ218" s="74"/>
-      <c r="CR218" s="74"/>
-      <c r="CS218" s="74"/>
-      <c r="CT218" s="74"/>
-      <c r="CU218" s="74"/>
-      <c r="CV218" s="74"/>
-      <c r="CW218" s="74"/>
-      <c r="CX218" s="74"/>
-      <c r="CY218" s="74"/>
-      <c r="CZ218" s="74"/>
-      <c r="DA218" s="74"/>
-      <c r="DB218" s="74"/>
-      <c r="DC218" s="74"/>
-      <c r="DD218" s="74"/>
-      <c r="DE218" s="74"/>
-      <c r="DF218" s="74"/>
-      <c r="DG218" s="74"/>
-      <c r="DH218" s="74"/>
-      <c r="DI218" s="74"/>
-      <c r="DJ218" s="74"/>
-      <c r="DK218" s="74"/>
-      <c r="DL218" s="74"/>
-      <c r="DM218" s="74"/>
-    </row>
-    <row r="219" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A219" s="73">
+      <c r="K218" s="56"/>
+      <c r="L218" s="56"/>
+      <c r="M218" s="56"/>
+      <c r="N218" s="56"/>
+      <c r="O218" s="56"/>
+      <c r="P218" s="56"/>
+      <c r="Q218" s="56"/>
+      <c r="R218" s="56"/>
+      <c r="S218" s="56"/>
+      <c r="T218" s="56"/>
+      <c r="U218" s="56"/>
+      <c r="V218" s="56"/>
+      <c r="W218" s="56"/>
+      <c r="X218" s="56"/>
+      <c r="Y218" s="56"/>
+      <c r="Z218" s="56"/>
+      <c r="AA218" s="56"/>
+      <c r="AB218" s="56"/>
+      <c r="AC218" s="56"/>
+      <c r="AD218" s="56"/>
+      <c r="AE218" s="56"/>
+      <c r="AF218" s="56"/>
+      <c r="AG218" s="56"/>
+      <c r="AH218" s="56"/>
+      <c r="AI218" s="56"/>
+      <c r="AJ218" s="56"/>
+      <c r="AK218" s="56"/>
+      <c r="AL218" s="56"/>
+      <c r="AM218" s="56"/>
+      <c r="AN218" s="56"/>
+      <c r="AO218" s="56"/>
+      <c r="AP218" s="56"/>
+      <c r="AQ218" s="56"/>
+      <c r="AR218" s="56"/>
+      <c r="AS218" s="56"/>
+      <c r="AT218" s="56"/>
+      <c r="AU218" s="56"/>
+      <c r="AV218" s="56"/>
+      <c r="AW218" s="56"/>
+      <c r="AX218" s="56"/>
+      <c r="AY218" s="56"/>
+      <c r="AZ218" s="56"/>
+      <c r="BA218" s="56"/>
+      <c r="BB218" s="56"/>
+      <c r="BC218" s="56"/>
+      <c r="BD218" s="56"/>
+      <c r="BE218" s="56"/>
+      <c r="BF218" s="56"/>
+      <c r="BG218" s="56"/>
+      <c r="BH218" s="56"/>
+      <c r="BI218" s="56"/>
+      <c r="BJ218" s="56"/>
+      <c r="BK218" s="56"/>
+      <c r="BL218" s="56"/>
+      <c r="BM218" s="56"/>
+      <c r="BN218" s="56"/>
+      <c r="BO218" s="56"/>
+      <c r="BP218" s="56"/>
+      <c r="BQ218" s="56"/>
+      <c r="BR218" s="56"/>
+      <c r="BS218" s="56"/>
+      <c r="BT218" s="56"/>
+      <c r="BU218" s="56"/>
+      <c r="BV218" s="56"/>
+      <c r="BW218" s="56"/>
+      <c r="BX218" s="56"/>
+      <c r="BY218" s="56"/>
+      <c r="BZ218" s="56"/>
+      <c r="CA218" s="56"/>
+      <c r="CB218" s="56"/>
+      <c r="CC218" s="56"/>
+      <c r="CD218" s="56"/>
+      <c r="CE218" s="56"/>
+      <c r="CF218" s="56"/>
+      <c r="CG218" s="56"/>
+      <c r="CH218" s="56"/>
+      <c r="CI218" s="56"/>
+      <c r="CJ218" s="56"/>
+      <c r="CK218" s="56"/>
+      <c r="CL218" s="56"/>
+      <c r="CM218" s="56"/>
+      <c r="CN218" s="56"/>
+      <c r="CO218" s="56"/>
+      <c r="CP218" s="56"/>
+      <c r="CQ218" s="56"/>
+      <c r="CR218" s="56"/>
+      <c r="CS218" s="56"/>
+      <c r="CT218" s="56"/>
+      <c r="CU218" s="56"/>
+      <c r="CV218" s="56"/>
+      <c r="CW218" s="56"/>
+      <c r="CX218" s="56"/>
+      <c r="CY218" s="56"/>
+      <c r="CZ218" s="56"/>
+      <c r="DA218" s="56"/>
+      <c r="DB218" s="56"/>
+      <c r="DC218" s="56"/>
+      <c r="DD218" s="56"/>
+      <c r="DE218" s="56"/>
+      <c r="DF218" s="56"/>
+      <c r="DG218" s="56"/>
+      <c r="DH218" s="56"/>
+      <c r="DI218" s="56"/>
+      <c r="DJ218" s="56"/>
+      <c r="DK218" s="56"/>
+      <c r="DL218" s="56"/>
+      <c r="DM218" s="56"/>
+    </row>
+    <row r="219" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A219" s="55">
         <v>2026</v>
       </c>
-      <c r="B219" s="73" t="s">
+      <c r="B219" s="55" t="s">
         <v>989</v>
       </c>
-      <c r="C219" s="73" t="s">
+      <c r="C219" s="55" t="s">
         <v>625</v>
       </c>
-      <c r="E219" s="73" t="s">
+      <c r="E219" s="55" t="s">
         <v>472</v>
       </c>
-      <c r="F219" s="73" t="s">
+      <c r="F219" s="55" t="s">
         <v>583</v>
       </c>
-      <c r="K219" s="74"/>
-      <c r="L219" s="74"/>
-      <c r="M219" s="74"/>
-      <c r="N219" s="74"/>
-      <c r="O219" s="74"/>
-      <c r="P219" s="74"/>
-      <c r="Q219" s="74"/>
-      <c r="R219" s="74"/>
-      <c r="S219" s="74"/>
-      <c r="T219" s="74"/>
-      <c r="U219" s="74"/>
-      <c r="V219" s="74"/>
-      <c r="W219" s="74"/>
-      <c r="X219" s="74"/>
-      <c r="Y219" s="74"/>
-      <c r="Z219" s="74"/>
-      <c r="AA219" s="74"/>
-      <c r="AB219" s="74"/>
-      <c r="AC219" s="74"/>
-      <c r="AD219" s="74"/>
-      <c r="AE219" s="74"/>
-      <c r="AF219" s="74"/>
-      <c r="AG219" s="74"/>
-      <c r="AH219" s="74"/>
-      <c r="AI219" s="74"/>
-      <c r="AJ219" s="74"/>
-      <c r="AK219" s="74"/>
-      <c r="AL219" s="74"/>
-      <c r="AM219" s="74"/>
-      <c r="AN219" s="74"/>
-      <c r="AO219" s="74"/>
-      <c r="AP219" s="74"/>
-      <c r="AQ219" s="74"/>
-      <c r="AR219" s="74"/>
-      <c r="AS219" s="74"/>
-      <c r="AT219" s="74"/>
-      <c r="AU219" s="74"/>
-      <c r="AV219" s="74"/>
-      <c r="AW219" s="74"/>
-      <c r="AX219" s="74"/>
-      <c r="AY219" s="74"/>
-      <c r="AZ219" s="74"/>
-      <c r="BA219" s="74"/>
-      <c r="BB219" s="74"/>
-      <c r="BC219" s="74"/>
-      <c r="BD219" s="74"/>
-      <c r="BE219" s="74"/>
-      <c r="BF219" s="74"/>
-      <c r="BG219" s="74"/>
-      <c r="BH219" s="74"/>
-      <c r="BI219" s="74"/>
-      <c r="BJ219" s="74"/>
-      <c r="BK219" s="74"/>
-      <c r="BL219" s="74"/>
-      <c r="BM219" s="74"/>
-      <c r="BN219" s="74"/>
-      <c r="BO219" s="74"/>
-      <c r="BP219" s="74"/>
-      <c r="BQ219" s="74"/>
-      <c r="BR219" s="74"/>
-      <c r="BS219" s="74"/>
-      <c r="BT219" s="74"/>
-      <c r="BU219" s="74"/>
-      <c r="BV219" s="74"/>
-      <c r="BW219" s="74"/>
-      <c r="BX219" s="74"/>
-      <c r="BY219" s="74"/>
-      <c r="BZ219" s="74"/>
-      <c r="CA219" s="74"/>
-      <c r="CB219" s="74"/>
-      <c r="CC219" s="74"/>
-      <c r="CD219" s="74"/>
-      <c r="CE219" s="74"/>
-      <c r="CF219" s="74"/>
-      <c r="CG219" s="74"/>
-      <c r="CH219" s="74"/>
-      <c r="CI219" s="74"/>
-      <c r="CJ219" s="74"/>
-      <c r="CK219" s="74"/>
-      <c r="CL219" s="74"/>
-      <c r="CM219" s="74"/>
-      <c r="CN219" s="74"/>
-      <c r="CO219" s="74"/>
-      <c r="CP219" s="74"/>
-      <c r="CQ219" s="74"/>
-      <c r="CR219" s="74"/>
-      <c r="CS219" s="74"/>
-      <c r="CT219" s="74"/>
-      <c r="CU219" s="74"/>
-      <c r="CV219" s="74"/>
-      <c r="CW219" s="74"/>
-      <c r="CX219" s="74"/>
-      <c r="CY219" s="74"/>
-      <c r="CZ219" s="74"/>
-      <c r="DA219" s="74"/>
-      <c r="DB219" s="74"/>
-      <c r="DC219" s="74"/>
-      <c r="DD219" s="74"/>
-      <c r="DE219" s="74"/>
-      <c r="DF219" s="74"/>
-      <c r="DG219" s="74"/>
-      <c r="DH219" s="74"/>
-      <c r="DI219" s="74"/>
-      <c r="DJ219" s="74"/>
-      <c r="DK219" s="74"/>
-      <c r="DL219" s="74"/>
-      <c r="DM219" s="74"/>
-    </row>
-    <row r="220" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A220" s="73">
+      <c r="K219" s="56"/>
+      <c r="L219" s="56"/>
+      <c r="M219" s="56"/>
+      <c r="N219" s="56"/>
+      <c r="O219" s="56"/>
+      <c r="P219" s="56"/>
+      <c r="Q219" s="56"/>
+      <c r="R219" s="56"/>
+      <c r="S219" s="56"/>
+      <c r="T219" s="56"/>
+      <c r="U219" s="56"/>
+      <c r="V219" s="56"/>
+      <c r="W219" s="56"/>
+      <c r="X219" s="56"/>
+      <c r="Y219" s="56"/>
+      <c r="Z219" s="56"/>
+      <c r="AA219" s="56"/>
+      <c r="AB219" s="56"/>
+      <c r="AC219" s="56"/>
+      <c r="AD219" s="56"/>
+      <c r="AE219" s="56"/>
+      <c r="AF219" s="56"/>
+      <c r="AG219" s="56"/>
+      <c r="AH219" s="56"/>
+      <c r="AI219" s="56"/>
+      <c r="AJ219" s="56"/>
+      <c r="AK219" s="56"/>
+      <c r="AL219" s="56"/>
+      <c r="AM219" s="56"/>
+      <c r="AN219" s="56"/>
+      <c r="AO219" s="56"/>
+      <c r="AP219" s="56"/>
+      <c r="AQ219" s="56"/>
+      <c r="AR219" s="56"/>
+      <c r="AS219" s="56"/>
+      <c r="AT219" s="56"/>
+      <c r="AU219" s="56"/>
+      <c r="AV219" s="56"/>
+      <c r="AW219" s="56"/>
+      <c r="AX219" s="56"/>
+      <c r="AY219" s="56"/>
+      <c r="AZ219" s="56"/>
+      <c r="BA219" s="56"/>
+      <c r="BB219" s="56"/>
+      <c r="BC219" s="56"/>
+      <c r="BD219" s="56"/>
+      <c r="BE219" s="56"/>
+      <c r="BF219" s="56"/>
+      <c r="BG219" s="56"/>
+      <c r="BH219" s="56"/>
+      <c r="BI219" s="56"/>
+      <c r="BJ219" s="56"/>
+      <c r="BK219" s="56"/>
+      <c r="BL219" s="56"/>
+      <c r="BM219" s="56"/>
+      <c r="BN219" s="56"/>
+      <c r="BO219" s="56"/>
+      <c r="BP219" s="56"/>
+      <c r="BQ219" s="56"/>
+      <c r="BR219" s="56"/>
+      <c r="BS219" s="56"/>
+      <c r="BT219" s="56"/>
+      <c r="BU219" s="56"/>
+      <c r="BV219" s="56"/>
+      <c r="BW219" s="56"/>
+      <c r="BX219" s="56"/>
+      <c r="BY219" s="56"/>
+      <c r="BZ219" s="56"/>
+      <c r="CA219" s="56"/>
+      <c r="CB219" s="56"/>
+      <c r="CC219" s="56"/>
+      <c r="CD219" s="56"/>
+      <c r="CE219" s="56"/>
+      <c r="CF219" s="56"/>
+      <c r="CG219" s="56"/>
+      <c r="CH219" s="56"/>
+      <c r="CI219" s="56"/>
+      <c r="CJ219" s="56"/>
+      <c r="CK219" s="56"/>
+      <c r="CL219" s="56"/>
+      <c r="CM219" s="56"/>
+      <c r="CN219" s="56"/>
+      <c r="CO219" s="56"/>
+      <c r="CP219" s="56"/>
+      <c r="CQ219" s="56"/>
+      <c r="CR219" s="56"/>
+      <c r="CS219" s="56"/>
+      <c r="CT219" s="56"/>
+      <c r="CU219" s="56"/>
+      <c r="CV219" s="56"/>
+      <c r="CW219" s="56"/>
+      <c r="CX219" s="56"/>
+      <c r="CY219" s="56"/>
+      <c r="CZ219" s="56"/>
+      <c r="DA219" s="56"/>
+      <c r="DB219" s="56"/>
+      <c r="DC219" s="56"/>
+      <c r="DD219" s="56"/>
+      <c r="DE219" s="56"/>
+      <c r="DF219" s="56"/>
+      <c r="DG219" s="56"/>
+      <c r="DH219" s="56"/>
+      <c r="DI219" s="56"/>
+      <c r="DJ219" s="56"/>
+      <c r="DK219" s="56"/>
+      <c r="DL219" s="56"/>
+      <c r="DM219" s="56"/>
+    </row>
+    <row r="220" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A220" s="55">
         <v>2026</v>
       </c>
-      <c r="B220" s="73" t="s">
+      <c r="B220" s="55" t="s">
         <v>990</v>
       </c>
-      <c r="C220" s="73" t="s">
+      <c r="C220" s="55" t="s">
         <v>991</v>
       </c>
-      <c r="E220" s="73" t="s">
+      <c r="E220" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="F220" s="73" t="s">
+      <c r="F220" s="55" t="s">
         <v>495</v>
       </c>
-      <c r="K220" s="74"/>
-      <c r="L220" s="74"/>
-      <c r="M220" s="74"/>
-      <c r="N220" s="74"/>
-      <c r="O220" s="74"/>
-      <c r="P220" s="74"/>
-      <c r="Q220" s="74"/>
-      <c r="R220" s="74"/>
-      <c r="S220" s="74"/>
-      <c r="T220" s="74"/>
-      <c r="U220" s="74"/>
-      <c r="V220" s="74"/>
-      <c r="W220" s="74"/>
-      <c r="X220" s="74"/>
-      <c r="Y220" s="74"/>
-      <c r="Z220" s="74"/>
-      <c r="AA220" s="74"/>
-      <c r="AB220" s="74"/>
-      <c r="AC220" s="74"/>
-      <c r="AD220" s="74"/>
-      <c r="AE220" s="74"/>
-      <c r="AF220" s="74"/>
-      <c r="AG220" s="74"/>
-      <c r="AH220" s="74"/>
-      <c r="AI220" s="74"/>
-      <c r="AJ220" s="74"/>
-      <c r="AK220" s="74"/>
-      <c r="AL220" s="74"/>
-      <c r="AM220" s="74"/>
-      <c r="AN220" s="74"/>
-      <c r="AO220" s="74"/>
-      <c r="AP220" s="74"/>
-      <c r="AQ220" s="74"/>
-      <c r="AR220" s="74"/>
-      <c r="AS220" s="74"/>
-      <c r="AT220" s="74"/>
-      <c r="AU220" s="74"/>
-      <c r="AV220" s="74"/>
-      <c r="AW220" s="74"/>
-      <c r="AX220" s="74"/>
-      <c r="AY220" s="74"/>
-      <c r="AZ220" s="74"/>
-      <c r="BA220" s="74"/>
-      <c r="BB220" s="74"/>
-      <c r="BC220" s="74"/>
-      <c r="BD220" s="74"/>
-      <c r="BE220" s="74"/>
-      <c r="BF220" s="74"/>
-      <c r="BG220" s="74"/>
-      <c r="BH220" s="74"/>
-      <c r="BI220" s="74"/>
-      <c r="BJ220" s="74"/>
-      <c r="BK220" s="74"/>
-      <c r="BL220" s="74"/>
-      <c r="BM220" s="74"/>
-      <c r="BN220" s="74"/>
-      <c r="BO220" s="74"/>
-      <c r="BP220" s="74"/>
-      <c r="BQ220" s="74"/>
-      <c r="BR220" s="74"/>
-      <c r="BS220" s="74"/>
-      <c r="BT220" s="74"/>
-      <c r="BU220" s="74"/>
-      <c r="BV220" s="74"/>
-      <c r="BW220" s="74"/>
-      <c r="BX220" s="74"/>
-      <c r="BY220" s="74"/>
-      <c r="BZ220" s="74"/>
-      <c r="CA220" s="74"/>
-      <c r="CB220" s="74"/>
-      <c r="CC220" s="74"/>
-      <c r="CD220" s="74"/>
-      <c r="CE220" s="74"/>
-      <c r="CF220" s="74"/>
-      <c r="CG220" s="74"/>
-      <c r="CH220" s="74"/>
-      <c r="CI220" s="74"/>
-      <c r="CJ220" s="74"/>
-      <c r="CK220" s="74"/>
-      <c r="CL220" s="74"/>
-      <c r="CM220" s="74"/>
-      <c r="CN220" s="74"/>
-      <c r="CO220" s="74"/>
-      <c r="CP220" s="74"/>
-      <c r="CQ220" s="74"/>
-      <c r="CR220" s="74"/>
-      <c r="CS220" s="74"/>
-      <c r="CT220" s="74"/>
-      <c r="CU220" s="74"/>
-      <c r="CV220" s="74"/>
-      <c r="CW220" s="74"/>
-      <c r="CX220" s="74"/>
-      <c r="CY220" s="74"/>
-      <c r="CZ220" s="74"/>
-      <c r="DA220" s="74"/>
-      <c r="DB220" s="74"/>
-      <c r="DC220" s="74"/>
-      <c r="DD220" s="74"/>
-      <c r="DE220" s="74"/>
-      <c r="DF220" s="74"/>
-      <c r="DG220" s="74"/>
-      <c r="DH220" s="74"/>
-      <c r="DI220" s="74"/>
-      <c r="DJ220" s="74"/>
-      <c r="DK220" s="74"/>
-      <c r="DL220" s="74"/>
-      <c r="DM220" s="74"/>
-    </row>
-    <row r="221" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A221" s="73">
+      <c r="K220" s="56"/>
+      <c r="L220" s="56"/>
+      <c r="M220" s="56"/>
+      <c r="N220" s="56"/>
+      <c r="O220" s="56"/>
+      <c r="P220" s="56"/>
+      <c r="Q220" s="56"/>
+      <c r="R220" s="56"/>
+      <c r="S220" s="56"/>
+      <c r="T220" s="56"/>
+      <c r="U220" s="56"/>
+      <c r="V220" s="56"/>
+      <c r="W220" s="56"/>
+      <c r="X220" s="56"/>
+      <c r="Y220" s="56"/>
+      <c r="Z220" s="56"/>
+      <c r="AA220" s="56"/>
+      <c r="AB220" s="56"/>
+      <c r="AC220" s="56"/>
+      <c r="AD220" s="56"/>
+      <c r="AE220" s="56"/>
+      <c r="AF220" s="56"/>
+      <c r="AG220" s="56"/>
+      <c r="AH220" s="56"/>
+      <c r="AI220" s="56"/>
+      <c r="AJ220" s="56"/>
+      <c r="AK220" s="56"/>
+      <c r="AL220" s="56"/>
+      <c r="AM220" s="56"/>
+      <c r="AN220" s="56"/>
+      <c r="AO220" s="56"/>
+      <c r="AP220" s="56"/>
+      <c r="AQ220" s="56"/>
+      <c r="AR220" s="56"/>
+      <c r="AS220" s="56"/>
+      <c r="AT220" s="56"/>
+      <c r="AU220" s="56"/>
+      <c r="AV220" s="56"/>
+      <c r="AW220" s="56"/>
+      <c r="AX220" s="56"/>
+      <c r="AY220" s="56"/>
+      <c r="AZ220" s="56"/>
+      <c r="BA220" s="56"/>
+      <c r="BB220" s="56"/>
+      <c r="BC220" s="56"/>
+      <c r="BD220" s="56"/>
+      <c r="BE220" s="56"/>
+      <c r="BF220" s="56"/>
+      <c r="BG220" s="56"/>
+      <c r="BH220" s="56"/>
+      <c r="BI220" s="56"/>
+      <c r="BJ220" s="56"/>
+      <c r="BK220" s="56"/>
+      <c r="BL220" s="56"/>
+      <c r="BM220" s="56"/>
+      <c r="BN220" s="56"/>
+      <c r="BO220" s="56"/>
+      <c r="BP220" s="56"/>
+      <c r="BQ220" s="56"/>
+      <c r="BR220" s="56"/>
+      <c r="BS220" s="56"/>
+      <c r="BT220" s="56"/>
+      <c r="BU220" s="56"/>
+      <c r="BV220" s="56"/>
+      <c r="BW220" s="56"/>
+      <c r="BX220" s="56"/>
+      <c r="BY220" s="56"/>
+      <c r="BZ220" s="56"/>
+      <c r="CA220" s="56"/>
+      <c r="CB220" s="56"/>
+      <c r="CC220" s="56"/>
+      <c r="CD220" s="56"/>
+      <c r="CE220" s="56"/>
+      <c r="CF220" s="56"/>
+      <c r="CG220" s="56"/>
+      <c r="CH220" s="56"/>
+      <c r="CI220" s="56"/>
+      <c r="CJ220" s="56"/>
+      <c r="CK220" s="56"/>
+      <c r="CL220" s="56"/>
+      <c r="CM220" s="56"/>
+      <c r="CN220" s="56"/>
+      <c r="CO220" s="56"/>
+      <c r="CP220" s="56"/>
+      <c r="CQ220" s="56"/>
+      <c r="CR220" s="56"/>
+      <c r="CS220" s="56"/>
+      <c r="CT220" s="56"/>
+      <c r="CU220" s="56"/>
+      <c r="CV220" s="56"/>
+      <c r="CW220" s="56"/>
+      <c r="CX220" s="56"/>
+      <c r="CY220" s="56"/>
+      <c r="CZ220" s="56"/>
+      <c r="DA220" s="56"/>
+      <c r="DB220" s="56"/>
+      <c r="DC220" s="56"/>
+      <c r="DD220" s="56"/>
+      <c r="DE220" s="56"/>
+      <c r="DF220" s="56"/>
+      <c r="DG220" s="56"/>
+      <c r="DH220" s="56"/>
+      <c r="DI220" s="56"/>
+      <c r="DJ220" s="56"/>
+      <c r="DK220" s="56"/>
+      <c r="DL220" s="56"/>
+      <c r="DM220" s="56"/>
+    </row>
+    <row r="221" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A221" s="55">
         <v>2026</v>
       </c>
-      <c r="B221" s="73" t="s">
+      <c r="B221" s="55" t="s">
         <v>992</v>
       </c>
-      <c r="C221" s="73" t="s">
+      <c r="C221" s="55" t="s">
         <v>993</v>
       </c>
-      <c r="E221" s="73" t="s">
+      <c r="E221" s="55" t="s">
         <v>182</v>
       </c>
-      <c r="F221" s="73" t="s">
+      <c r="F221" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="K221" s="74"/>
-      <c r="L221" s="74"/>
-      <c r="M221" s="74"/>
-      <c r="N221" s="74"/>
-      <c r="O221" s="74"/>
-      <c r="P221" s="74"/>
-      <c r="Q221" s="74"/>
-      <c r="R221" s="74"/>
-      <c r="S221" s="74"/>
-      <c r="T221" s="74"/>
-      <c r="U221" s="74"/>
-      <c r="V221" s="74"/>
-      <c r="W221" s="74"/>
-      <c r="X221" s="74"/>
-      <c r="Y221" s="74"/>
-      <c r="Z221" s="74"/>
-      <c r="AA221" s="74"/>
-      <c r="AB221" s="74"/>
-      <c r="AC221" s="74"/>
-      <c r="AD221" s="74"/>
-      <c r="AE221" s="74"/>
-      <c r="AF221" s="74"/>
-      <c r="AG221" s="74"/>
-      <c r="AH221" s="74"/>
-      <c r="AI221" s="74"/>
-      <c r="AJ221" s="74"/>
-      <c r="AK221" s="74"/>
-      <c r="AL221" s="74"/>
-      <c r="AM221" s="74"/>
-      <c r="AN221" s="74"/>
-      <c r="AO221" s="74"/>
-      <c r="AP221" s="74"/>
-      <c r="AQ221" s="74"/>
-      <c r="AR221" s="74"/>
-      <c r="AS221" s="74"/>
-      <c r="AT221" s="74"/>
-      <c r="AU221" s="74"/>
-      <c r="AV221" s="74"/>
-      <c r="AW221" s="74"/>
-      <c r="AX221" s="74"/>
-      <c r="AY221" s="74"/>
-      <c r="AZ221" s="74"/>
-      <c r="BA221" s="74"/>
-      <c r="BB221" s="74"/>
-      <c r="BC221" s="74"/>
-      <c r="BD221" s="74"/>
-      <c r="BE221" s="74"/>
-      <c r="BF221" s="74"/>
-      <c r="BG221" s="74"/>
-      <c r="BH221" s="74"/>
-      <c r="BI221" s="74"/>
-      <c r="BJ221" s="74"/>
-      <c r="BK221" s="74"/>
-      <c r="BL221" s="74"/>
-      <c r="BM221" s="74"/>
-      <c r="BN221" s="74"/>
-      <c r="BO221" s="74"/>
-      <c r="BP221" s="74"/>
-      <c r="BQ221" s="74"/>
-      <c r="BR221" s="74"/>
-      <c r="BS221" s="74"/>
-      <c r="BT221" s="74"/>
-      <c r="BU221" s="74"/>
-      <c r="BV221" s="74"/>
-      <c r="BW221" s="74"/>
-      <c r="BX221" s="74"/>
-      <c r="BY221" s="74"/>
-      <c r="BZ221" s="74"/>
-      <c r="CA221" s="74"/>
-      <c r="CB221" s="74"/>
-      <c r="CC221" s="74"/>
-      <c r="CD221" s="74"/>
-      <c r="CE221" s="74"/>
-      <c r="CF221" s="74"/>
-      <c r="CG221" s="74"/>
-      <c r="CH221" s="74"/>
-      <c r="CI221" s="74"/>
-      <c r="CJ221" s="74"/>
-      <c r="CK221" s="74"/>
-      <c r="CL221" s="74"/>
-      <c r="CM221" s="74"/>
-      <c r="CN221" s="74"/>
-      <c r="CO221" s="74"/>
-      <c r="CP221" s="74"/>
-      <c r="CQ221" s="74"/>
-      <c r="CR221" s="74"/>
-      <c r="CS221" s="74"/>
-      <c r="CT221" s="74"/>
-      <c r="CU221" s="74"/>
-      <c r="CV221" s="74"/>
-      <c r="CW221" s="74"/>
-      <c r="CX221" s="74"/>
-      <c r="CY221" s="74"/>
-      <c r="CZ221" s="74"/>
-      <c r="DA221" s="74"/>
-      <c r="DB221" s="74"/>
-      <c r="DC221" s="74"/>
-      <c r="DD221" s="74"/>
-      <c r="DE221" s="74"/>
-      <c r="DF221" s="74"/>
-      <c r="DG221" s="74"/>
-      <c r="DH221" s="74"/>
-      <c r="DI221" s="74"/>
-      <c r="DJ221" s="74"/>
-      <c r="DK221" s="74"/>
-      <c r="DL221" s="74"/>
-      <c r="DM221" s="74"/>
-    </row>
-    <row r="222" spans="1:117" s="73" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A222" s="73">
+      <c r="K221" s="56"/>
+      <c r="L221" s="56"/>
+      <c r="M221" s="56"/>
+      <c r="N221" s="56"/>
+      <c r="O221" s="56"/>
+      <c r="P221" s="56"/>
+      <c r="Q221" s="56"/>
+      <c r="R221" s="56"/>
+      <c r="S221" s="56"/>
+      <c r="T221" s="56"/>
+      <c r="U221" s="56"/>
+      <c r="V221" s="56"/>
+      <c r="W221" s="56"/>
+      <c r="X221" s="56"/>
+      <c r="Y221" s="56"/>
+      <c r="Z221" s="56"/>
+      <c r="AA221" s="56"/>
+      <c r="AB221" s="56"/>
+      <c r="AC221" s="56"/>
+      <c r="AD221" s="56"/>
+      <c r="AE221" s="56"/>
+      <c r="AF221" s="56"/>
+      <c r="AG221" s="56"/>
+      <c r="AH221" s="56"/>
+      <c r="AI221" s="56"/>
+      <c r="AJ221" s="56"/>
+      <c r="AK221" s="56"/>
+      <c r="AL221" s="56"/>
+      <c r="AM221" s="56"/>
+      <c r="AN221" s="56"/>
+      <c r="AO221" s="56"/>
+      <c r="AP221" s="56"/>
+      <c r="AQ221" s="56"/>
+      <c r="AR221" s="56"/>
+      <c r="AS221" s="56"/>
+      <c r="AT221" s="56"/>
+      <c r="AU221" s="56"/>
+      <c r="AV221" s="56"/>
+      <c r="AW221" s="56"/>
+      <c r="AX221" s="56"/>
+      <c r="AY221" s="56"/>
+      <c r="AZ221" s="56"/>
+      <c r="BA221" s="56"/>
+      <c r="BB221" s="56"/>
+      <c r="BC221" s="56"/>
+      <c r="BD221" s="56"/>
+      <c r="BE221" s="56"/>
+      <c r="BF221" s="56"/>
+      <c r="BG221" s="56"/>
+      <c r="BH221" s="56"/>
+      <c r="BI221" s="56"/>
+      <c r="BJ221" s="56"/>
+      <c r="BK221" s="56"/>
+      <c r="BL221" s="56"/>
+      <c r="BM221" s="56"/>
+      <c r="BN221" s="56"/>
+      <c r="BO221" s="56"/>
+      <c r="BP221" s="56"/>
+      <c r="BQ221" s="56"/>
+      <c r="BR221" s="56"/>
+      <c r="BS221" s="56"/>
+      <c r="BT221" s="56"/>
+      <c r="BU221" s="56"/>
+      <c r="BV221" s="56"/>
+      <c r="BW221" s="56"/>
+      <c r="BX221" s="56"/>
+      <c r="BY221" s="56"/>
+      <c r="BZ221" s="56"/>
+      <c r="CA221" s="56"/>
+      <c r="CB221" s="56"/>
+      <c r="CC221" s="56"/>
+      <c r="CD221" s="56"/>
+      <c r="CE221" s="56"/>
+      <c r="CF221" s="56"/>
+      <c r="CG221" s="56"/>
+      <c r="CH221" s="56"/>
+      <c r="CI221" s="56"/>
+      <c r="CJ221" s="56"/>
+      <c r="CK221" s="56"/>
+      <c r="CL221" s="56"/>
+      <c r="CM221" s="56"/>
+      <c r="CN221" s="56"/>
+      <c r="CO221" s="56"/>
+      <c r="CP221" s="56"/>
+      <c r="CQ221" s="56"/>
+      <c r="CR221" s="56"/>
+      <c r="CS221" s="56"/>
+      <c r="CT221" s="56"/>
+      <c r="CU221" s="56"/>
+      <c r="CV221" s="56"/>
+      <c r="CW221" s="56"/>
+      <c r="CX221" s="56"/>
+      <c r="CY221" s="56"/>
+      <c r="CZ221" s="56"/>
+      <c r="DA221" s="56"/>
+      <c r="DB221" s="56"/>
+      <c r="DC221" s="56"/>
+      <c r="DD221" s="56"/>
+      <c r="DE221" s="56"/>
+      <c r="DF221" s="56"/>
+      <c r="DG221" s="56"/>
+      <c r="DH221" s="56"/>
+      <c r="DI221" s="56"/>
+      <c r="DJ221" s="56"/>
+      <c r="DK221" s="56"/>
+      <c r="DL221" s="56"/>
+      <c r="DM221" s="56"/>
+    </row>
+    <row r="222" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A222" s="55">
         <v>2026</v>
       </c>
-      <c r="B222" s="73" t="s">
+      <c r="B222" s="55" t="s">
         <v>995</v>
       </c>
-      <c r="C222" s="73" t="s">
+      <c r="C222" s="55" t="s">
         <v>996</v>
       </c>
-      <c r="E222" s="73" t="s">
+      <c r="E222" s="55" t="s">
         <v>766</v>
       </c>
-      <c r="F222" s="73" t="s">
+      <c r="F222" s="55" t="s">
         <v>994</v>
       </c>
-      <c r="K222" s="74"/>
-      <c r="L222" s="74"/>
-      <c r="M222" s="74"/>
-      <c r="N222" s="74"/>
-      <c r="O222" s="74"/>
-      <c r="P222" s="74"/>
-      <c r="Q222" s="74"/>
-      <c r="R222" s="74"/>
-      <c r="S222" s="74"/>
-      <c r="T222" s="74"/>
-      <c r="U222" s="74"/>
-      <c r="V222" s="74"/>
-      <c r="W222" s="74"/>
-      <c r="X222" s="74"/>
-      <c r="Y222" s="74"/>
-      <c r="Z222" s="74"/>
-      <c r="AA222" s="74"/>
-      <c r="AB222" s="74"/>
-      <c r="AC222" s="74"/>
-      <c r="AD222" s="74"/>
-      <c r="AE222" s="74"/>
-      <c r="AF222" s="74"/>
-      <c r="AG222" s="74"/>
-      <c r="AH222" s="74"/>
-      <c r="AI222" s="74"/>
-      <c r="AJ222" s="74"/>
-      <c r="AK222" s="74"/>
-      <c r="AL222" s="74"/>
-      <c r="AM222" s="74"/>
-      <c r="AN222" s="74"/>
-      <c r="AO222" s="74"/>
-      <c r="AP222" s="74"/>
-      <c r="AQ222" s="74"/>
-      <c r="AR222" s="74"/>
-      <c r="AS222" s="74"/>
-      <c r="AT222" s="74"/>
-      <c r="AU222" s="74"/>
-      <c r="AV222" s="74"/>
-      <c r="AW222" s="74"/>
-      <c r="AX222" s="74"/>
-      <c r="AY222" s="74"/>
-      <c r="AZ222" s="74"/>
-      <c r="BA222" s="74"/>
-      <c r="BB222" s="74"/>
-      <c r="BC222" s="74"/>
-      <c r="BD222" s="74"/>
-      <c r="BE222" s="74"/>
-      <c r="BF222" s="74"/>
-      <c r="BG222" s="74"/>
-      <c r="BH222" s="74"/>
-      <c r="BI222" s="74"/>
-      <c r="BJ222" s="74"/>
-      <c r="BK222" s="74"/>
-      <c r="BL222" s="74"/>
-      <c r="BM222" s="74"/>
-      <c r="BN222" s="74"/>
-      <c r="BO222" s="74"/>
-      <c r="BP222" s="74"/>
-      <c r="BQ222" s="74"/>
-      <c r="BR222" s="74"/>
-      <c r="BS222" s="74"/>
-      <c r="BT222" s="74"/>
-      <c r="BU222" s="74"/>
-      <c r="BV222" s="74"/>
-      <c r="BW222" s="74"/>
-      <c r="BX222" s="74"/>
-      <c r="BY222" s="74"/>
-      <c r="BZ222" s="74"/>
-      <c r="CA222" s="74"/>
-      <c r="CB222" s="74"/>
-      <c r="CC222" s="74"/>
-      <c r="CD222" s="74"/>
-      <c r="CE222" s="74"/>
-      <c r="CF222" s="74"/>
-      <c r="CG222" s="74"/>
-      <c r="CH222" s="74"/>
-      <c r="CI222" s="74"/>
-      <c r="CJ222" s="74"/>
-      <c r="CK222" s="74"/>
-      <c r="CL222" s="74"/>
-      <c r="CM222" s="74"/>
-      <c r="CN222" s="74"/>
-      <c r="CO222" s="74"/>
-      <c r="CP222" s="74"/>
-      <c r="CQ222" s="74"/>
-      <c r="CR222" s="74"/>
-      <c r="CS222" s="74"/>
-      <c r="CT222" s="74"/>
-      <c r="CU222" s="74"/>
-      <c r="CV222" s="74"/>
-      <c r="CW222" s="74"/>
-      <c r="CX222" s="74"/>
-      <c r="CY222" s="74"/>
-      <c r="CZ222" s="74"/>
-      <c r="DA222" s="74"/>
-      <c r="DB222" s="74"/>
-      <c r="DC222" s="74"/>
-      <c r="DD222" s="74"/>
-      <c r="DE222" s="74"/>
-      <c r="DF222" s="74"/>
-      <c r="DG222" s="74"/>
-      <c r="DH222" s="74"/>
-      <c r="DI222" s="74"/>
-      <c r="DJ222" s="74"/>
-      <c r="DK222" s="74"/>
-      <c r="DL222" s="74"/>
-      <c r="DM222" s="74"/>
-    </row>
-    <row r="223" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A223" s="73">
+      <c r="K222" s="56"/>
+      <c r="L222" s="56"/>
+      <c r="M222" s="56"/>
+      <c r="N222" s="56"/>
+      <c r="O222" s="56"/>
+      <c r="P222" s="56"/>
+      <c r="Q222" s="56"/>
+      <c r="R222" s="56"/>
+      <c r="S222" s="56"/>
+      <c r="T222" s="56"/>
+      <c r="U222" s="56"/>
+      <c r="V222" s="56"/>
+      <c r="W222" s="56"/>
+      <c r="X222" s="56"/>
+      <c r="Y222" s="56"/>
+      <c r="Z222" s="56"/>
+      <c r="AA222" s="56"/>
+      <c r="AB222" s="56"/>
+      <c r="AC222" s="56"/>
+      <c r="AD222" s="56"/>
+      <c r="AE222" s="56"/>
+      <c r="AF222" s="56"/>
+      <c r="AG222" s="56"/>
+      <c r="AH222" s="56"/>
+      <c r="AI222" s="56"/>
+      <c r="AJ222" s="56"/>
+      <c r="AK222" s="56"/>
+      <c r="AL222" s="56"/>
+      <c r="AM222" s="56"/>
+      <c r="AN222" s="56"/>
+      <c r="AO222" s="56"/>
+      <c r="AP222" s="56"/>
+      <c r="AQ222" s="56"/>
+      <c r="AR222" s="56"/>
+      <c r="AS222" s="56"/>
+      <c r="AT222" s="56"/>
+      <c r="AU222" s="56"/>
+      <c r="AV222" s="56"/>
+      <c r="AW222" s="56"/>
+      <c r="AX222" s="56"/>
+      <c r="AY222" s="56"/>
+      <c r="AZ222" s="56"/>
+      <c r="BA222" s="56"/>
+      <c r="BB222" s="56"/>
+      <c r="BC222" s="56"/>
+      <c r="BD222" s="56"/>
+      <c r="BE222" s="56"/>
+      <c r="BF222" s="56"/>
+      <c r="BG222" s="56"/>
+      <c r="BH222" s="56"/>
+      <c r="BI222" s="56"/>
+      <c r="BJ222" s="56"/>
+      <c r="BK222" s="56"/>
+      <c r="BL222" s="56"/>
+      <c r="BM222" s="56"/>
+      <c r="BN222" s="56"/>
+      <c r="BO222" s="56"/>
+      <c r="BP222" s="56"/>
+      <c r="BQ222" s="56"/>
+      <c r="BR222" s="56"/>
+      <c r="BS222" s="56"/>
+      <c r="BT222" s="56"/>
+      <c r="BU222" s="56"/>
+      <c r="BV222" s="56"/>
+      <c r="BW222" s="56"/>
+      <c r="BX222" s="56"/>
+      <c r="BY222" s="56"/>
+      <c r="BZ222" s="56"/>
+      <c r="CA222" s="56"/>
+      <c r="CB222" s="56"/>
+      <c r="CC222" s="56"/>
+      <c r="CD222" s="56"/>
+      <c r="CE222" s="56"/>
+      <c r="CF222" s="56"/>
+      <c r="CG222" s="56"/>
+      <c r="CH222" s="56"/>
+      <c r="CI222" s="56"/>
+      <c r="CJ222" s="56"/>
+      <c r="CK222" s="56"/>
+      <c r="CL222" s="56"/>
+      <c r="CM222" s="56"/>
+      <c r="CN222" s="56"/>
+      <c r="CO222" s="56"/>
+      <c r="CP222" s="56"/>
+      <c r="CQ222" s="56"/>
+      <c r="CR222" s="56"/>
+      <c r="CS222" s="56"/>
+      <c r="CT222" s="56"/>
+      <c r="CU222" s="56"/>
+      <c r="CV222" s="56"/>
+      <c r="CW222" s="56"/>
+      <c r="CX222" s="56"/>
+      <c r="CY222" s="56"/>
+      <c r="CZ222" s="56"/>
+      <c r="DA222" s="56"/>
+      <c r="DB222" s="56"/>
+      <c r="DC222" s="56"/>
+      <c r="DD222" s="56"/>
+      <c r="DE222" s="56"/>
+      <c r="DF222" s="56"/>
+      <c r="DG222" s="56"/>
+      <c r="DH222" s="56"/>
+      <c r="DI222" s="56"/>
+      <c r="DJ222" s="56"/>
+      <c r="DK222" s="56"/>
+      <c r="DL222" s="56"/>
+      <c r="DM222" s="56"/>
+    </row>
+    <row r="223" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A223" s="55">
         <v>2026</v>
       </c>
-      <c r="B223" s="73" t="s">
+      <c r="B223" s="55" t="s">
         <v>997</v>
       </c>
-      <c r="C223" s="73" t="s">
+      <c r="C223" s="55" t="s">
         <v>998</v>
       </c>
-      <c r="E223" s="73" t="s">
+      <c r="E223" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="F223" s="73" t="s">
+      <c r="F223" s="55" t="s">
         <v>468</v>
       </c>
-      <c r="K223" s="74"/>
-      <c r="L223" s="74"/>
-      <c r="M223" s="74"/>
-      <c r="N223" s="74"/>
-      <c r="O223" s="74"/>
-      <c r="P223" s="74"/>
-      <c r="Q223" s="74"/>
-      <c r="R223" s="74"/>
-      <c r="S223" s="74"/>
-      <c r="T223" s="74"/>
-      <c r="U223" s="74"/>
-      <c r="V223" s="74"/>
-      <c r="W223" s="74"/>
-      <c r="X223" s="74"/>
-      <c r="Y223" s="74"/>
-      <c r="Z223" s="74"/>
-      <c r="AA223" s="74"/>
-      <c r="AB223" s="74"/>
-      <c r="AC223" s="74"/>
-      <c r="AD223" s="74"/>
-      <c r="AE223" s="74"/>
-      <c r="AF223" s="74"/>
-      <c r="AG223" s="74"/>
-      <c r="AH223" s="74"/>
-      <c r="AI223" s="74"/>
-      <c r="AJ223" s="74"/>
-      <c r="AK223" s="74"/>
-      <c r="AL223" s="74"/>
-      <c r="AM223" s="74"/>
-      <c r="AN223" s="74"/>
-      <c r="AO223" s="74"/>
-      <c r="AP223" s="74"/>
-      <c r="AQ223" s="74"/>
-      <c r="AR223" s="74"/>
-      <c r="AS223" s="74"/>
-      <c r="AT223" s="74"/>
-      <c r="AU223" s="74"/>
-      <c r="AV223" s="74"/>
-      <c r="AW223" s="74"/>
-      <c r="AX223" s="74"/>
-      <c r="AY223" s="74"/>
-      <c r="AZ223" s="74"/>
-      <c r="BA223" s="74"/>
-      <c r="BB223" s="74"/>
-      <c r="BC223" s="74"/>
-      <c r="BD223" s="74"/>
-      <c r="BE223" s="74"/>
-      <c r="BF223" s="74"/>
-      <c r="BG223" s="74"/>
-      <c r="BH223" s="74"/>
-      <c r="BI223" s="74"/>
-      <c r="BJ223" s="74"/>
-      <c r="BK223" s="74"/>
-      <c r="BL223" s="74"/>
-      <c r="BM223" s="74"/>
-      <c r="BN223" s="74"/>
-      <c r="BO223" s="74"/>
-      <c r="BP223" s="74"/>
-      <c r="BQ223" s="74"/>
-      <c r="BR223" s="74"/>
-      <c r="BS223" s="74"/>
-      <c r="BT223" s="74"/>
-      <c r="BU223" s="74"/>
-      <c r="BV223" s="74"/>
-      <c r="BW223" s="74"/>
-      <c r="BX223" s="74"/>
-      <c r="BY223" s="74"/>
-      <c r="BZ223" s="74"/>
-      <c r="CA223" s="74"/>
-      <c r="CB223" s="74"/>
-      <c r="CC223" s="74"/>
-      <c r="CD223" s="74"/>
-      <c r="CE223" s="74"/>
-      <c r="CF223" s="74"/>
-      <c r="CG223" s="74"/>
-      <c r="CH223" s="74"/>
-      <c r="CI223" s="74"/>
-      <c r="CJ223" s="74"/>
-      <c r="CK223" s="74"/>
-      <c r="CL223" s="74"/>
-      <c r="CM223" s="74"/>
-      <c r="CN223" s="74"/>
-      <c r="CO223" s="74"/>
-      <c r="CP223" s="74"/>
-      <c r="CQ223" s="74"/>
-      <c r="CR223" s="74"/>
-      <c r="CS223" s="74"/>
-      <c r="CT223" s="74"/>
-      <c r="CU223" s="74"/>
-      <c r="CV223" s="74"/>
-      <c r="CW223" s="74"/>
-      <c r="CX223" s="74"/>
-      <c r="CY223" s="74"/>
-      <c r="CZ223" s="74"/>
-      <c r="DA223" s="74"/>
-      <c r="DB223" s="74"/>
-      <c r="DC223" s="74"/>
-      <c r="DD223" s="74"/>
-      <c r="DE223" s="74"/>
-      <c r="DF223" s="74"/>
-      <c r="DG223" s="74"/>
-      <c r="DH223" s="74"/>
-      <c r="DI223" s="74"/>
-      <c r="DJ223" s="74"/>
-      <c r="DK223" s="74"/>
-      <c r="DL223" s="74"/>
-      <c r="DM223" s="74"/>
-    </row>
-    <row r="224" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A224" s="73">
+      <c r="K223" s="56"/>
+      <c r="L223" s="56"/>
+      <c r="M223" s="56"/>
+      <c r="N223" s="56"/>
+      <c r="O223" s="56"/>
+      <c r="P223" s="56"/>
+      <c r="Q223" s="56"/>
+      <c r="R223" s="56"/>
+      <c r="S223" s="56"/>
+      <c r="T223" s="56"/>
+      <c r="U223" s="56"/>
+      <c r="V223" s="56"/>
+      <c r="W223" s="56"/>
+      <c r="X223" s="56"/>
+      <c r="Y223" s="56"/>
+      <c r="Z223" s="56"/>
+      <c r="AA223" s="56"/>
+      <c r="AB223" s="56"/>
+      <c r="AC223" s="56"/>
+      <c r="AD223" s="56"/>
+      <c r="AE223" s="56"/>
+      <c r="AF223" s="56"/>
+      <c r="AG223" s="56"/>
+      <c r="AH223" s="56"/>
+      <c r="AI223" s="56"/>
+      <c r="AJ223" s="56"/>
+      <c r="AK223" s="56"/>
+      <c r="AL223" s="56"/>
+      <c r="AM223" s="56"/>
+      <c r="AN223" s="56"/>
+      <c r="AO223" s="56"/>
+      <c r="AP223" s="56"/>
+      <c r="AQ223" s="56"/>
+      <c r="AR223" s="56"/>
+      <c r="AS223" s="56"/>
+      <c r="AT223" s="56"/>
+      <c r="AU223" s="56"/>
+      <c r="AV223" s="56"/>
+      <c r="AW223" s="56"/>
+      <c r="AX223" s="56"/>
+      <c r="AY223" s="56"/>
+      <c r="AZ223" s="56"/>
+      <c r="BA223" s="56"/>
+      <c r="BB223" s="56"/>
+      <c r="BC223" s="56"/>
+      <c r="BD223" s="56"/>
+      <c r="BE223" s="56"/>
+      <c r="BF223" s="56"/>
+      <c r="BG223" s="56"/>
+      <c r="BH223" s="56"/>
+      <c r="BI223" s="56"/>
+      <c r="BJ223" s="56"/>
+      <c r="BK223" s="56"/>
+      <c r="BL223" s="56"/>
+      <c r="BM223" s="56"/>
+      <c r="BN223" s="56"/>
+      <c r="BO223" s="56"/>
+      <c r="BP223" s="56"/>
+      <c r="BQ223" s="56"/>
+      <c r="BR223" s="56"/>
+      <c r="BS223" s="56"/>
+      <c r="BT223" s="56"/>
+      <c r="BU223" s="56"/>
+      <c r="BV223" s="56"/>
+      <c r="BW223" s="56"/>
+      <c r="BX223" s="56"/>
+      <c r="BY223" s="56"/>
+      <c r="BZ223" s="56"/>
+      <c r="CA223" s="56"/>
+      <c r="CB223" s="56"/>
+      <c r="CC223" s="56"/>
+      <c r="CD223" s="56"/>
+      <c r="CE223" s="56"/>
+      <c r="CF223" s="56"/>
+      <c r="CG223" s="56"/>
+      <c r="CH223" s="56"/>
+      <c r="CI223" s="56"/>
+      <c r="CJ223" s="56"/>
+      <c r="CK223" s="56"/>
+      <c r="CL223" s="56"/>
+      <c r="CM223" s="56"/>
+      <c r="CN223" s="56"/>
+      <c r="CO223" s="56"/>
+      <c r="CP223" s="56"/>
+      <c r="CQ223" s="56"/>
+      <c r="CR223" s="56"/>
+      <c r="CS223" s="56"/>
+      <c r="CT223" s="56"/>
+      <c r="CU223" s="56"/>
+      <c r="CV223" s="56"/>
+      <c r="CW223" s="56"/>
+      <c r="CX223" s="56"/>
+      <c r="CY223" s="56"/>
+      <c r="CZ223" s="56"/>
+      <c r="DA223" s="56"/>
+      <c r="DB223" s="56"/>
+      <c r="DC223" s="56"/>
+      <c r="DD223" s="56"/>
+      <c r="DE223" s="56"/>
+      <c r="DF223" s="56"/>
+      <c r="DG223" s="56"/>
+      <c r="DH223" s="56"/>
+      <c r="DI223" s="56"/>
+      <c r="DJ223" s="56"/>
+      <c r="DK223" s="56"/>
+      <c r="DL223" s="56"/>
+      <c r="DM223" s="56"/>
+    </row>
+    <row r="224" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A224" s="55">
         <v>2026</v>
       </c>
-      <c r="B224" s="73" t="s">
+      <c r="B224" s="55" t="s">
         <v>999</v>
       </c>
-      <c r="C224" s="73" t="s">
+      <c r="C224" s="55" t="s">
         <v>596</v>
       </c>
       <c r="E224" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="F224" s="73" t="s">
+      <c r="F224" s="55" t="s">
         <v>182</v>
       </c>
-      <c r="K224" s="74"/>
-      <c r="L224" s="74"/>
-      <c r="M224" s="74"/>
-      <c r="N224" s="74"/>
-      <c r="O224" s="74"/>
-      <c r="P224" s="74"/>
-      <c r="Q224" s="74"/>
-      <c r="R224" s="74"/>
-      <c r="S224" s="74"/>
-      <c r="T224" s="74"/>
-      <c r="U224" s="74"/>
-      <c r="V224" s="74"/>
-      <c r="W224" s="74"/>
-      <c r="X224" s="74"/>
-      <c r="Y224" s="74"/>
-      <c r="Z224" s="74"/>
-      <c r="AA224" s="74"/>
-      <c r="AB224" s="74"/>
-      <c r="AC224" s="74"/>
-      <c r="AD224" s="74"/>
-      <c r="AE224" s="74"/>
-      <c r="AF224" s="74"/>
-      <c r="AG224" s="74"/>
-      <c r="AH224" s="74"/>
-      <c r="AI224" s="74"/>
-      <c r="AJ224" s="74"/>
-      <c r="AK224" s="74"/>
-      <c r="AL224" s="74"/>
-      <c r="AM224" s="74"/>
-      <c r="AN224" s="74"/>
-      <c r="AO224" s="74"/>
-      <c r="AP224" s="74"/>
-      <c r="AQ224" s="74"/>
-      <c r="AR224" s="74"/>
-      <c r="AS224" s="74"/>
-      <c r="AT224" s="74"/>
-      <c r="AU224" s="74"/>
-      <c r="AV224" s="74"/>
-      <c r="AW224" s="74"/>
-      <c r="AX224" s="74"/>
-      <c r="AY224" s="74"/>
-      <c r="AZ224" s="74"/>
-      <c r="BA224" s="74"/>
-      <c r="BB224" s="74"/>
-      <c r="BC224" s="74"/>
-      <c r="BD224" s="74"/>
-      <c r="BE224" s="74"/>
-      <c r="BF224" s="74"/>
-      <c r="BG224" s="74"/>
-      <c r="BH224" s="74"/>
-      <c r="BI224" s="74"/>
-      <c r="BJ224" s="74"/>
-      <c r="BK224" s="74"/>
-      <c r="BL224" s="74"/>
-      <c r="BM224" s="74"/>
-      <c r="BN224" s="74"/>
-      <c r="BO224" s="74"/>
-      <c r="BP224" s="74"/>
-      <c r="BQ224" s="74"/>
-      <c r="BR224" s="74"/>
-      <c r="BS224" s="74"/>
-      <c r="BT224" s="74"/>
-      <c r="BU224" s="74"/>
-      <c r="BV224" s="74"/>
-      <c r="BW224" s="74"/>
-      <c r="BX224" s="74"/>
-      <c r="BY224" s="74"/>
-      <c r="BZ224" s="74"/>
-      <c r="CA224" s="74"/>
-      <c r="CB224" s="74"/>
-      <c r="CC224" s="74"/>
-      <c r="CD224" s="74"/>
-      <c r="CE224" s="74"/>
-      <c r="CF224" s="74"/>
-      <c r="CG224" s="74"/>
-      <c r="CH224" s="74"/>
-      <c r="CI224" s="74"/>
-      <c r="CJ224" s="74"/>
-      <c r="CK224" s="74"/>
-      <c r="CL224" s="74"/>
-      <c r="CM224" s="74"/>
-      <c r="CN224" s="74"/>
-      <c r="CO224" s="74"/>
-      <c r="CP224" s="74"/>
-      <c r="CQ224" s="74"/>
-      <c r="CR224" s="74"/>
-      <c r="CS224" s="74"/>
-      <c r="CT224" s="74"/>
-      <c r="CU224" s="74"/>
-      <c r="CV224" s="74"/>
-      <c r="CW224" s="74"/>
-      <c r="CX224" s="74"/>
-      <c r="CY224" s="74"/>
-      <c r="CZ224" s="74"/>
-      <c r="DA224" s="74"/>
-      <c r="DB224" s="74"/>
-      <c r="DC224" s="74"/>
-      <c r="DD224" s="74"/>
-      <c r="DE224" s="74"/>
-      <c r="DF224" s="74"/>
-      <c r="DG224" s="74"/>
-      <c r="DH224" s="74"/>
-      <c r="DI224" s="74"/>
-      <c r="DJ224" s="74"/>
-      <c r="DK224" s="74"/>
-      <c r="DL224" s="74"/>
-      <c r="DM224" s="74"/>
-    </row>
-    <row r="225" spans="1:117" s="73" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A225" s="73">
+      <c r="K224" s="56"/>
+      <c r="L224" s="56"/>
+      <c r="M224" s="56"/>
+      <c r="N224" s="56"/>
+      <c r="O224" s="56"/>
+      <c r="P224" s="56"/>
+      <c r="Q224" s="56"/>
+      <c r="R224" s="56"/>
+      <c r="S224" s="56"/>
+      <c r="T224" s="56"/>
+      <c r="U224" s="56"/>
+      <c r="V224" s="56"/>
+      <c r="W224" s="56"/>
+      <c r="X224" s="56"/>
+      <c r="Y224" s="56"/>
+      <c r="Z224" s="56"/>
+      <c r="AA224" s="56"/>
+      <c r="AB224" s="56"/>
+      <c r="AC224" s="56"/>
+      <c r="AD224" s="56"/>
+      <c r="AE224" s="56"/>
+      <c r="AF224" s="56"/>
+      <c r="AG224" s="56"/>
+      <c r="AH224" s="56"/>
+      <c r="AI224" s="56"/>
+      <c r="AJ224" s="56"/>
+      <c r="AK224" s="56"/>
+      <c r="AL224" s="56"/>
+      <c r="AM224" s="56"/>
+      <c r="AN224" s="56"/>
+      <c r="AO224" s="56"/>
+      <c r="AP224" s="56"/>
+      <c r="AQ224" s="56"/>
+      <c r="AR224" s="56"/>
+      <c r="AS224" s="56"/>
+      <c r="AT224" s="56"/>
+      <c r="AU224" s="56"/>
+      <c r="AV224" s="56"/>
+      <c r="AW224" s="56"/>
+      <c r="AX224" s="56"/>
+      <c r="AY224" s="56"/>
+      <c r="AZ224" s="56"/>
+      <c r="BA224" s="56"/>
+      <c r="BB224" s="56"/>
+      <c r="BC224" s="56"/>
+      <c r="BD224" s="56"/>
+      <c r="BE224" s="56"/>
+      <c r="BF224" s="56"/>
+      <c r="BG224" s="56"/>
+      <c r="BH224" s="56"/>
+      <c r="BI224" s="56"/>
+      <c r="BJ224" s="56"/>
+      <c r="BK224" s="56"/>
+      <c r="BL224" s="56"/>
+      <c r="BM224" s="56"/>
+      <c r="BN224" s="56"/>
+      <c r="BO224" s="56"/>
+      <c r="BP224" s="56"/>
+      <c r="BQ224" s="56"/>
+      <c r="BR224" s="56"/>
+      <c r="BS224" s="56"/>
+      <c r="BT224" s="56"/>
+      <c r="BU224" s="56"/>
+      <c r="BV224" s="56"/>
+      <c r="BW224" s="56"/>
+      <c r="BX224" s="56"/>
+      <c r="BY224" s="56"/>
+      <c r="BZ224" s="56"/>
+      <c r="CA224" s="56"/>
+      <c r="CB224" s="56"/>
+      <c r="CC224" s="56"/>
+      <c r="CD224" s="56"/>
+      <c r="CE224" s="56"/>
+      <c r="CF224" s="56"/>
+      <c r="CG224" s="56"/>
+      <c r="CH224" s="56"/>
+      <c r="CI224" s="56"/>
+      <c r="CJ224" s="56"/>
+      <c r="CK224" s="56"/>
+      <c r="CL224" s="56"/>
+      <c r="CM224" s="56"/>
+      <c r="CN224" s="56"/>
+      <c r="CO224" s="56"/>
+      <c r="CP224" s="56"/>
+      <c r="CQ224" s="56"/>
+      <c r="CR224" s="56"/>
+      <c r="CS224" s="56"/>
+      <c r="CT224" s="56"/>
+      <c r="CU224" s="56"/>
+      <c r="CV224" s="56"/>
+      <c r="CW224" s="56"/>
+      <c r="CX224" s="56"/>
+      <c r="CY224" s="56"/>
+      <c r="CZ224" s="56"/>
+      <c r="DA224" s="56"/>
+      <c r="DB224" s="56"/>
+      <c r="DC224" s="56"/>
+      <c r="DD224" s="56"/>
+      <c r="DE224" s="56"/>
+      <c r="DF224" s="56"/>
+      <c r="DG224" s="56"/>
+      <c r="DH224" s="56"/>
+      <c r="DI224" s="56"/>
+      <c r="DJ224" s="56"/>
+      <c r="DK224" s="56"/>
+      <c r="DL224" s="56"/>
+      <c r="DM224" s="56"/>
+    </row>
+    <row r="225" spans="1:117" s="55" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A225" s="55">
         <v>2026</v>
       </c>
-      <c r="B225" s="73" t="s">
+      <c r="B225" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="C225" s="73" t="s">
+      <c r="C225" s="55" t="s">
         <v>1000</v>
       </c>
-      <c r="E225" s="73" t="s">
+      <c r="E225" s="55" t="s">
         <v>182</v>
       </c>
-      <c r="F225" s="73" t="s">
+      <c r="F225" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="K225" s="74"/>
-      <c r="L225" s="74"/>
-      <c r="M225" s="74"/>
-      <c r="N225" s="74"/>
-      <c r="O225" s="74"/>
-      <c r="P225" s="74"/>
-      <c r="Q225" s="74"/>
-      <c r="R225" s="74"/>
-      <c r="S225" s="74"/>
-      <c r="T225" s="74"/>
-      <c r="U225" s="74"/>
-      <c r="V225" s="74"/>
-      <c r="W225" s="74"/>
-      <c r="X225" s="74"/>
-      <c r="Y225" s="74"/>
-      <c r="Z225" s="74"/>
-      <c r="AA225" s="74"/>
-      <c r="AB225" s="74"/>
-      <c r="AC225" s="74"/>
-      <c r="AD225" s="74"/>
-      <c r="AE225" s="74"/>
-      <c r="AF225" s="74"/>
-      <c r="AG225" s="74"/>
-      <c r="AH225" s="74"/>
-      <c r="AI225" s="74"/>
-      <c r="AJ225" s="74"/>
-      <c r="AK225" s="74"/>
-      <c r="AL225" s="74"/>
-      <c r="AM225" s="74"/>
-      <c r="AN225" s="74"/>
-      <c r="AO225" s="74"/>
-      <c r="AP225" s="74"/>
-      <c r="AQ225" s="74"/>
-      <c r="AR225" s="74"/>
-      <c r="AS225" s="74"/>
-      <c r="AT225" s="74"/>
-      <c r="AU225" s="74"/>
-      <c r="AV225" s="74"/>
-      <c r="AW225" s="74"/>
-      <c r="AX225" s="74"/>
-      <c r="AY225" s="74"/>
-      <c r="AZ225" s="74"/>
-      <c r="BA225" s="74"/>
-      <c r="BB225" s="74"/>
-      <c r="BC225" s="74"/>
-      <c r="BD225" s="74"/>
-      <c r="BE225" s="74"/>
-      <c r="BF225" s="74"/>
-      <c r="BG225" s="74"/>
-      <c r="BH225" s="74"/>
-      <c r="BI225" s="74"/>
-      <c r="BJ225" s="74"/>
-      <c r="BK225" s="74"/>
-      <c r="BL225" s="74"/>
-      <c r="BM225" s="74"/>
-      <c r="BN225" s="74"/>
-      <c r="BO225" s="74"/>
-      <c r="BP225" s="74"/>
-      <c r="BQ225" s="74"/>
-      <c r="BR225" s="74"/>
-      <c r="BS225" s="74"/>
-      <c r="BT225" s="74"/>
-      <c r="BU225" s="74"/>
-      <c r="BV225" s="74"/>
-      <c r="BW225" s="74"/>
-      <c r="BX225" s="74"/>
-      <c r="BY225" s="74"/>
-      <c r="BZ225" s="74"/>
-      <c r="CA225" s="74"/>
-      <c r="CB225" s="74"/>
-      <c r="CC225" s="74"/>
-      <c r="CD225" s="74"/>
-      <c r="CE225" s="74"/>
-      <c r="CF225" s="74"/>
-      <c r="CG225" s="74"/>
-      <c r="CH225" s="74"/>
-      <c r="CI225" s="74"/>
-      <c r="CJ225" s="74"/>
-      <c r="CK225" s="74"/>
-      <c r="CL225" s="74"/>
-      <c r="CM225" s="74"/>
-      <c r="CN225" s="74"/>
-      <c r="CO225" s="74"/>
-      <c r="CP225" s="74"/>
-      <c r="CQ225" s="74"/>
-      <c r="CR225" s="74"/>
-      <c r="CS225" s="74"/>
-      <c r="CT225" s="74"/>
-      <c r="CU225" s="74"/>
-      <c r="CV225" s="74"/>
-      <c r="CW225" s="74"/>
-      <c r="CX225" s="74"/>
-      <c r="CY225" s="74"/>
-      <c r="CZ225" s="74"/>
-      <c r="DA225" s="74"/>
-      <c r="DB225" s="74"/>
-      <c r="DC225" s="74"/>
-      <c r="DD225" s="74"/>
-      <c r="DE225" s="74"/>
-      <c r="DF225" s="74"/>
-      <c r="DG225" s="74"/>
-      <c r="DH225" s="74"/>
-      <c r="DI225" s="74"/>
-      <c r="DJ225" s="74"/>
-      <c r="DK225" s="74"/>
-      <c r="DL225" s="74"/>
-      <c r="DM225" s="74"/>
-    </row>
-    <row r="226" spans="1:117" s="73" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="K226" s="74"/>
-      <c r="L226" s="74"/>
-      <c r="M226" s="74"/>
-      <c r="N226" s="74"/>
-      <c r="O226" s="74"/>
-      <c r="P226" s="74"/>
-      <c r="Q226" s="74"/>
-      <c r="R226" s="74"/>
-      <c r="S226" s="74"/>
-      <c r="T226" s="74"/>
-      <c r="U226" s="74"/>
-      <c r="V226" s="74"/>
-      <c r="W226" s="74"/>
-      <c r="X226" s="74"/>
-      <c r="Y226" s="74"/>
-      <c r="Z226" s="74"/>
-      <c r="AA226" s="74"/>
-      <c r="AB226" s="74"/>
-      <c r="AC226" s="74"/>
-      <c r="AD226" s="74"/>
-      <c r="AE226" s="74"/>
-      <c r="AF226" s="74"/>
-      <c r="AG226" s="74"/>
-      <c r="AH226" s="74"/>
-      <c r="AI226" s="74"/>
-      <c r="AJ226" s="74"/>
-      <c r="AK226" s="74"/>
-      <c r="AL226" s="74"/>
-      <c r="AM226" s="74"/>
-      <c r="AN226" s="74"/>
-      <c r="AO226" s="74"/>
-      <c r="AP226" s="74"/>
-      <c r="AQ226" s="74"/>
-      <c r="AR226" s="74"/>
-      <c r="AS226" s="74"/>
-      <c r="AT226" s="74"/>
-      <c r="AU226" s="74"/>
-      <c r="AV226" s="74"/>
-      <c r="AW226" s="74"/>
-      <c r="AX226" s="74"/>
-      <c r="AY226" s="74"/>
-      <c r="AZ226" s="74"/>
-      <c r="BA226" s="74"/>
-      <c r="BB226" s="74"/>
-      <c r="BC226" s="74"/>
-      <c r="BD226" s="74"/>
-      <c r="BE226" s="74"/>
-      <c r="BF226" s="74"/>
-      <c r="BG226" s="74"/>
-      <c r="BH226" s="74"/>
-      <c r="BI226" s="74"/>
-      <c r="BJ226" s="74"/>
-      <c r="BK226" s="74"/>
-      <c r="BL226" s="74"/>
-      <c r="BM226" s="74"/>
-      <c r="BN226" s="74"/>
-      <c r="BO226" s="74"/>
-      <c r="BP226" s="74"/>
-      <c r="BQ226" s="74"/>
-      <c r="BR226" s="74"/>
-      <c r="BS226" s="74"/>
-      <c r="BT226" s="74"/>
-      <c r="BU226" s="74"/>
-      <c r="BV226" s="74"/>
-      <c r="BW226" s="74"/>
-      <c r="BX226" s="74"/>
-      <c r="BY226" s="74"/>
-      <c r="BZ226" s="74"/>
-      <c r="CA226" s="74"/>
-      <c r="CB226" s="74"/>
-      <c r="CC226" s="74"/>
-      <c r="CD226" s="74"/>
-      <c r="CE226" s="74"/>
-      <c r="CF226" s="74"/>
-      <c r="CG226" s="74"/>
-      <c r="CH226" s="74"/>
-      <c r="CI226" s="74"/>
-      <c r="CJ226" s="74"/>
-      <c r="CK226" s="74"/>
-      <c r="CL226" s="74"/>
-      <c r="CM226" s="74"/>
-      <c r="CN226" s="74"/>
-      <c r="CO226" s="74"/>
-      <c r="CP226" s="74"/>
-      <c r="CQ226" s="74"/>
-      <c r="CR226" s="74"/>
-      <c r="CS226" s="74"/>
-      <c r="CT226" s="74"/>
-      <c r="CU226" s="74"/>
-      <c r="CV226" s="74"/>
-      <c r="CW226" s="74"/>
-      <c r="CX226" s="74"/>
-      <c r="CY226" s="74"/>
-      <c r="CZ226" s="74"/>
-      <c r="DA226" s="74"/>
-      <c r="DB226" s="74"/>
-      <c r="DC226" s="74"/>
-      <c r="DD226" s="74"/>
-      <c r="DE226" s="74"/>
-      <c r="DF226" s="74"/>
-      <c r="DG226" s="74"/>
-      <c r="DH226" s="74"/>
-      <c r="DI226" s="74"/>
-      <c r="DJ226" s="74"/>
-      <c r="DK226" s="74"/>
-      <c r="DL226" s="74"/>
-      <c r="DM226" s="74"/>
+      <c r="K225" s="56"/>
+      <c r="L225" s="56"/>
+      <c r="M225" s="56"/>
+      <c r="N225" s="56"/>
+      <c r="O225" s="56"/>
+      <c r="P225" s="56"/>
+      <c r="Q225" s="56"/>
+      <c r="R225" s="56"/>
+      <c r="S225" s="56"/>
+      <c r="T225" s="56"/>
+      <c r="U225" s="56"/>
+      <c r="V225" s="56"/>
+      <c r="W225" s="56"/>
+      <c r="X225" s="56"/>
+      <c r="Y225" s="56"/>
+      <c r="Z225" s="56"/>
+      <c r="AA225" s="56"/>
+      <c r="AB225" s="56"/>
+      <c r="AC225" s="56"/>
+      <c r="AD225" s="56"/>
+      <c r="AE225" s="56"/>
+      <c r="AF225" s="56"/>
+      <c r="AG225" s="56"/>
+      <c r="AH225" s="56"/>
+      <c r="AI225" s="56"/>
+      <c r="AJ225" s="56"/>
+      <c r="AK225" s="56"/>
+      <c r="AL225" s="56"/>
+      <c r="AM225" s="56"/>
+      <c r="AN225" s="56"/>
+      <c r="AO225" s="56"/>
+      <c r="AP225" s="56"/>
+      <c r="AQ225" s="56"/>
+      <c r="AR225" s="56"/>
+      <c r="AS225" s="56"/>
+      <c r="AT225" s="56"/>
+      <c r="AU225" s="56"/>
+      <c r="AV225" s="56"/>
+      <c r="AW225" s="56"/>
+      <c r="AX225" s="56"/>
+      <c r="AY225" s="56"/>
+      <c r="AZ225" s="56"/>
+      <c r="BA225" s="56"/>
+      <c r="BB225" s="56"/>
+      <c r="BC225" s="56"/>
+      <c r="BD225" s="56"/>
+      <c r="BE225" s="56"/>
+      <c r="BF225" s="56"/>
+      <c r="BG225" s="56"/>
+      <c r="BH225" s="56"/>
+      <c r="BI225" s="56"/>
+      <c r="BJ225" s="56"/>
+      <c r="BK225" s="56"/>
+      <c r="BL225" s="56"/>
+      <c r="BM225" s="56"/>
+      <c r="BN225" s="56"/>
+      <c r="BO225" s="56"/>
+      <c r="BP225" s="56"/>
+      <c r="BQ225" s="56"/>
+      <c r="BR225" s="56"/>
+      <c r="BS225" s="56"/>
+      <c r="BT225" s="56"/>
+      <c r="BU225" s="56"/>
+      <c r="BV225" s="56"/>
+      <c r="BW225" s="56"/>
+      <c r="BX225" s="56"/>
+      <c r="BY225" s="56"/>
+      <c r="BZ225" s="56"/>
+      <c r="CA225" s="56"/>
+      <c r="CB225" s="56"/>
+      <c r="CC225" s="56"/>
+      <c r="CD225" s="56"/>
+      <c r="CE225" s="56"/>
+      <c r="CF225" s="56"/>
+      <c r="CG225" s="56"/>
+      <c r="CH225" s="56"/>
+      <c r="CI225" s="56"/>
+      <c r="CJ225" s="56"/>
+      <c r="CK225" s="56"/>
+      <c r="CL225" s="56"/>
+      <c r="CM225" s="56"/>
+      <c r="CN225" s="56"/>
+      <c r="CO225" s="56"/>
+      <c r="CP225" s="56"/>
+      <c r="CQ225" s="56"/>
+      <c r="CR225" s="56"/>
+      <c r="CS225" s="56"/>
+      <c r="CT225" s="56"/>
+      <c r="CU225" s="56"/>
+      <c r="CV225" s="56"/>
+      <c r="CW225" s="56"/>
+      <c r="CX225" s="56"/>
+      <c r="CY225" s="56"/>
+      <c r="CZ225" s="56"/>
+      <c r="DA225" s="56"/>
+      <c r="DB225" s="56"/>
+      <c r="DC225" s="56"/>
+      <c r="DD225" s="56"/>
+      <c r="DE225" s="56"/>
+      <c r="DF225" s="56"/>
+      <c r="DG225" s="56"/>
+      <c r="DH225" s="56"/>
+      <c r="DI225" s="56"/>
+      <c r="DJ225" s="56"/>
+      <c r="DK225" s="56"/>
+      <c r="DL225" s="56"/>
+      <c r="DM225" s="56"/>
+    </row>
+    <row r="226" spans="1:117" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="K226" s="56"/>
+      <c r="L226" s="56"/>
+      <c r="M226" s="56"/>
+      <c r="N226" s="56"/>
+      <c r="O226" s="56"/>
+      <c r="P226" s="56"/>
+      <c r="Q226" s="56"/>
+      <c r="R226" s="56"/>
+      <c r="S226" s="56"/>
+      <c r="T226" s="56"/>
+      <c r="U226" s="56"/>
+      <c r="V226" s="56"/>
+      <c r="W226" s="56"/>
+      <c r="X226" s="56"/>
+      <c r="Y226" s="56"/>
+      <c r="Z226" s="56"/>
+      <c r="AA226" s="56"/>
+      <c r="AB226" s="56"/>
+      <c r="AC226" s="56"/>
+      <c r="AD226" s="56"/>
+      <c r="AE226" s="56"/>
+      <c r="AF226" s="56"/>
+      <c r="AG226" s="56"/>
+      <c r="AH226" s="56"/>
+      <c r="AI226" s="56"/>
+      <c r="AJ226" s="56"/>
+      <c r="AK226" s="56"/>
+      <c r="AL226" s="56"/>
+      <c r="AM226" s="56"/>
+      <c r="AN226" s="56"/>
+      <c r="AO226" s="56"/>
+      <c r="AP226" s="56"/>
+      <c r="AQ226" s="56"/>
+      <c r="AR226" s="56"/>
+      <c r="AS226" s="56"/>
+      <c r="AT226" s="56"/>
+      <c r="AU226" s="56"/>
+      <c r="AV226" s="56"/>
+      <c r="AW226" s="56"/>
+      <c r="AX226" s="56"/>
+      <c r="AY226" s="56"/>
+      <c r="AZ226" s="56"/>
+      <c r="BA226" s="56"/>
+      <c r="BB226" s="56"/>
+      <c r="BC226" s="56"/>
+      <c r="BD226" s="56"/>
+      <c r="BE226" s="56"/>
+      <c r="BF226" s="56"/>
+      <c r="BG226" s="56"/>
+      <c r="BH226" s="56"/>
+      <c r="BI226" s="56"/>
+      <c r="BJ226" s="56"/>
+      <c r="BK226" s="56"/>
+      <c r="BL226" s="56"/>
+      <c r="BM226" s="56"/>
+      <c r="BN226" s="56"/>
+      <c r="BO226" s="56"/>
+      <c r="BP226" s="56"/>
+      <c r="BQ226" s="56"/>
+      <c r="BR226" s="56"/>
+      <c r="BS226" s="56"/>
+      <c r="BT226" s="56"/>
+      <c r="BU226" s="56"/>
+      <c r="BV226" s="56"/>
+      <c r="BW226" s="56"/>
+      <c r="BX226" s="56"/>
+      <c r="BY226" s="56"/>
+      <c r="BZ226" s="56"/>
+      <c r="CA226" s="56"/>
+      <c r="CB226" s="56"/>
+      <c r="CC226" s="56"/>
+      <c r="CD226" s="56"/>
+      <c r="CE226" s="56"/>
+      <c r="CF226" s="56"/>
+      <c r="CG226" s="56"/>
+      <c r="CH226" s="56"/>
+      <c r="CI226" s="56"/>
+      <c r="CJ226" s="56"/>
+      <c r="CK226" s="56"/>
+      <c r="CL226" s="56"/>
+      <c r="CM226" s="56"/>
+      <c r="CN226" s="56"/>
+      <c r="CO226" s="56"/>
+      <c r="CP226" s="56"/>
+      <c r="CQ226" s="56"/>
+      <c r="CR226" s="56"/>
+      <c r="CS226" s="56"/>
+      <c r="CT226" s="56"/>
+      <c r="CU226" s="56"/>
+      <c r="CV226" s="56"/>
+      <c r="CW226" s="56"/>
+      <c r="CX226" s="56"/>
+      <c r="CY226" s="56"/>
+      <c r="CZ226" s="56"/>
+      <c r="DA226" s="56"/>
+      <c r="DB226" s="56"/>
+      <c r="DC226" s="56"/>
+      <c r="DD226" s="56"/>
+      <c r="DE226" s="56"/>
+      <c r="DF226" s="56"/>
+      <c r="DG226" s="56"/>
+      <c r="DH226" s="56"/>
+      <c r="DI226" s="56"/>
+      <c r="DJ226" s="56"/>
+      <c r="DK226" s="56"/>
+      <c r="DL226" s="56"/>
+      <c r="DM226" s="56"/>
     </row>
     <row r="227" spans="1:117" x14ac:dyDescent="0.2">
-      <c r="A227" s="73"/>
+      <c r="A227" s="55"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -15906,8 +15909,8 @@
     <col min="4" max="16384" width="9.1640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="60" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="60" t="s">
+    <row r="1" spans="1:3" s="65" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>853</v>
       </c>
     </row>
@@ -16011,7 +16014,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="66" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="13" t="s">
@@ -16022,7 +16025,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="61"/>
+      <c r="A12" s="66"/>
       <c r="B12" s="13" t="s">
         <v>871</v>
       </c>
@@ -16031,7 +16034,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A13" s="61"/>
+      <c r="A13" s="66"/>
       <c r="B13" s="13" t="s">
         <v>873</v>
       </c>
@@ -16051,7 +16054,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="67" t="s">
         <v>877</v>
       </c>
       <c r="B15" s="13" t="s">
@@ -16062,7 +16065,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="63"/>
+      <c r="A16" s="68"/>
       <c r="B16" s="13" t="s">
         <v>880</v>
       </c>
@@ -16071,7 +16074,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="63"/>
+      <c r="A17" s="68"/>
       <c r="B17" s="13" t="s">
         <v>882</v>
       </c>
@@ -16080,7 +16083,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A18" s="63"/>
+      <c r="A18" s="68"/>
       <c r="B18" s="13" t="s">
         <v>884</v>
       </c>
@@ -16089,7 +16092,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="64"/>
+      <c r="A19" s="69"/>
       <c r="B19" s="13" t="s">
         <v>886</v>
       </c>
@@ -16175,7 +16178,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A27" s="68" t="s">
+      <c r="A27" s="73" t="s">
         <v>907</v>
       </c>
       <c r="B27" s="32" t="s">
@@ -16186,7 +16189,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A28" s="69"/>
+      <c r="A28" s="74"/>
       <c r="B28" s="52" t="s">
         <v>910</v>
       </c>
@@ -16195,7 +16198,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A29" s="70"/>
+      <c r="A29" s="75"/>
       <c r="B29" s="33" t="s">
         <v>912</v>
       </c>
@@ -16236,25 +16239,25 @@
       <c r="C33" s="14"/>
     </row>
     <row r="34" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="65" t="s">
+      <c r="A34" s="70" t="s">
         <v>919</v>
       </c>
-      <c r="B34" s="65"/>
-      <c r="C34" s="65"/>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
     </row>
     <row r="35" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="66" t="s">
+      <c r="A35" s="71" t="s">
         <v>920</v>
       </c>
-      <c r="B35" s="67"/>
-      <c r="C35" s="67"/>
+      <c r="B35" s="72"/>
+      <c r="C35" s="72"/>
     </row>
     <row r="36" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="59" t="s">
+      <c r="A36" s="64" t="s">
         <v>921</v>
       </c>
-      <c r="B36" s="59"/>
-      <c r="C36" s="59"/>
+      <c r="B36" s="64"/>
+      <c r="C36" s="64"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -16274,6 +16277,76 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="0b48997a-71d5-4c78-b23c-2d244392d80f">
+      <UserInfo>
+        <DisplayName>Salcedo, Ernesto (CDB)</DisplayName>
+        <AccountId>12</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Leppek, Noah</DisplayName>
+        <AccountId>11</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lohman, Chelsea</DisplayName>
+        <AccountId>18</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Corigliano, Michael</DisplayName>
+        <AccountId>19</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Griggs, Rocio</DisplayName>
+        <AccountId>20</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Heeschen, Ezra</DisplayName>
+        <AccountId>21</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Morse, Paul</DisplayName>
+        <AccountId>22</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lor, Billy</DisplayName>
+        <AccountId>23</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <Year xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580" xsi:nil="true"/>
+    <Chair xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Chair>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0b48997a-71d5-4c78-b23c-2d244392d80f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001D85B3B98401DE46ADFCC36F031FB8DB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6e246eeaec95f1c3563a9604188cbe35">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0b48997a-71d5-4c78-b23c-2d244392d80f" xmlns:ns3="0aa6ae91-60aa-4e93-b1be-e2f270f16580" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="840931b36835127a8d9177a1d8947058" ns2:_="" ns3:_="">
     <xsd:import namespace="0b48997a-71d5-4c78-b23c-2d244392d80f"/>
@@ -16524,77 +16597,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="0b48997a-71d5-4c78-b23c-2d244392d80f">
-      <UserInfo>
-        <DisplayName>Salcedo, Ernesto (CDB)</DisplayName>
-        <AccountId>12</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Leppek, Noah</DisplayName>
-        <AccountId>11</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lohman, Chelsea</DisplayName>
-        <AccountId>18</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Corigliano, Michael</DisplayName>
-        <AccountId>19</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Griggs, Rocio</DisplayName>
-        <AccountId>20</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Heeschen, Ezra</DisplayName>
-        <AccountId>21</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Morse, Paul</DisplayName>
-        <AccountId>22</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lor, Billy</DisplayName>
-        <AccountId>23</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <Year xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580" xsi:nil="true"/>
-    <Chair xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Chair>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0aa6ae91-60aa-4e93-b1be-e2f270f16580">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0b48997a-71d5-4c78-b23c-2d244392d80f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{434963E7-8327-4415-91CC-6F20EE0093BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC43AF2-F906-40F4-B939-3C31A42D720E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0b48997a-71d5-4c78-b23c-2d244392d80f"/>
+    <ds:schemaRef ds:uri="0aa6ae91-60aa-4e93-b1be-e2f270f16580"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DA3C789-3CF6-48B0-A044-3998A41365A2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16611,23 +16633,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC43AF2-F906-40F4-B939-3C31A42D720E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0b48997a-71d5-4c78-b23c-2d244392d80f"/>
-    <ds:schemaRef ds:uri="0aa6ae91-60aa-4e93-b1be-e2f270f16580"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{434963E7-8327-4415-91CC-6F20EE0093BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>